<commit_message>
구현: CAPL DLL Phase 1 ABI 기반 추가
- Win32/x86 M485E DLL과 CAPL_DLL_INFO4 기반 21개 API를 추가

- 독립 ABI Probe 및 CANalyzer CAPL Probe를 추가

- 빌드 구성과 개발 문서의 추적성 내용을 최신화
</commit_message>
<xml_diff>
--- a/docs/04_Traceability/Modbus485Emulator_Traceability_Matrix.xlsx
+++ b/docs/04_Traceability/Modbus485Emulator_Traceability_Matrix.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R212b4b9f9fc346ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="2" r:id="R6e9152ddd4134790"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R1a5ec813541b4c65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional Specs" sheetId="4" r:id="R7815105165a9498b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Components" sheetId="5" r:id="R484f93c31ef54859"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification Inputs" sheetId="6" r:id="R2753866374c4446a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R2b9ecc2e232c4856"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="2" r:id="R2ce999600d0f4252"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R59c595e390414e66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional Specs" sheetId="4" r:id="R3415fec85e8f41ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Components" sheetId="5" r:id="Re2d75cebc01843d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification Inputs" sheetId="6" r:id="Rce6cbd40336845a2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -110,7 +110,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -174,6 +174,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -569,7 +572,7 @@
         <x:v>Design Components</x:v>
       </x:c>
       <x:c r="E5" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -591,7 +594,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>0.9</x:v>
+        <x:v>0.10</x:v>
       </x:c>
       <x:c r="D7" s="11" t="str">
         <x:v>Requirements with Design</x:v>
@@ -619,7 +622,7 @@
         <x:v>Baseline Date</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-08-08</x:v>
+        <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
         <x:v>Test Case IDs</x:v>
@@ -775,7 +778,7 @@
     <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A1" s="21" t="str">
         <x:v>Requirement ID</x:v>
       </x:c>
@@ -786,7 +789,7 @@
         <x:v>Functional Specification ID</x:v>
       </x:c>
       <x:c r="D1" s="21" t="str">
-        <x:v>Design Component</x:v>
+        <x:v>Design Component ID / Name</x:v>
       </x:c>
       <x:c r="E1" s="21" t="str">
         <x:v>Verification Method</x:v>
@@ -801,7 +804,7 @@
         <x:v>Source Requirement IDs</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="32" customHeight="1">
+    <x:row r="2" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A2" s="22" t="str">
         <x:v>REQ-FUNC-001</x:v>
       </x:c>
@@ -812,7 +815,7 @@
         <x:v>FS-INIT-001</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>CAPL ABI Adapter; EmulatorContext</x:v>
+        <x:v>DC-01 CAPL ABI Adapter; DC-02 EmulatorContext</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
         <x:v>CANalyzer 9.x x86 DLL 로딩 및 중복 Context 시험</x:v>
@@ -825,7 +828,7 @@
         <x:v>FR-LIFE-009,016; IF-CTX-001~003,007</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="32" customHeight="1">
+    <x:row r="3" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A3" s="22" t="str">
         <x:v>REQ-FUNC-002</x:v>
       </x:c>
@@ -836,7 +839,7 @@
         <x:v>FS-LIFE-001,FS-LIFE-002,FS-LIFE-003</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>LifecycleController</x:v>
+        <x:v>DC-03 LifecycleController</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
         <x:v>Lifecycle 상태·Generation·Busy 처리 통합 시험</x:v>
@@ -849,7 +852,7 @@
         <x:v>FR-LIFE-010~015</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="32" customHeight="1">
+    <x:row r="4" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A4" s="22" t="str">
         <x:v>REQ-FUNC-003</x:v>
       </x:c>
@@ -860,7 +863,7 @@
         <x:v>FS-LIFE-003</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>LifecycleController</x:v>
+        <x:v>DC-03 LifecycleController</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
         <x:v>상태 전이 및 완료 결과 손실 방지 시험</x:v>
@@ -873,7 +876,7 @@
         <x:v>FR-LIFE-013~015; IF-CONST-003; IF-LSTAT-001~014</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="32" customHeight="1">
+    <x:row r="5" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A5" s="22" t="str">
         <x:v>REQ-FUNC-004</x:v>
       </x:c>
@@ -884,7 +887,7 @@
         <x:v>FS-LIFE-001</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>LifecycleController; Win32SerialPort; PortWorker</x:v>
+        <x:v>DC-03 LifecycleController; DC-09 Win32SerialPort; DC-10 PortWorker</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
         <x:v>두 번째 Port 실패 강제 및 전체 Rollback 시험</x:v>
@@ -897,7 +900,7 @@
         <x:v>FR-PORT-007~017</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="32" customHeight="1">
+    <x:row r="6" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A6" s="22" t="str">
         <x:v>REQ-FUNC-005</x:v>
       </x:c>
@@ -908,7 +911,7 @@
         <x:v>FS-LIFE-002</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
-        <x:v>LifecycleController; SnapshotService</x:v>
+        <x:v>DC-03 LifecycleController; DC-11 SnapshotService</x:v>
       </x:c>
       <x:c r="E6" s="9" t="str">
         <x:v>Disconnect/재Connect 데이터 보존 시험</x:v>
@@ -921,7 +924,7 @@
         <x:v>FR-LIFE-020,025,033</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="32" customHeight="1">
+    <x:row r="7" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A7" s="22" t="str">
         <x:v>REQ-FUNC-006</x:v>
       </x:c>
@@ -932,7 +935,7 @@
         <x:v>FS-LIFE-004</x:v>
       </x:c>
       <x:c r="D7" s="9" t="str">
-        <x:v>LifecycleController; PortWorker</x:v>
+        <x:v>DC-03 LifecycleController; DC-10 PortWorker</x:v>
       </x:c>
       <x:c r="E7" s="9" t="str">
         <x:v>USB 제거·복귀, 10회 실패 및 수동 복구 시험</x:v>
@@ -945,7 +948,7 @@
         <x:v>FR-LIFE-023~032</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="32" customHeight="1">
+    <x:row r="8" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A8" s="22" t="str">
         <x:v>REQ-FUNC-007</x:v>
       </x:c>
@@ -956,7 +959,7 @@
         <x:v>FS-LIFE-004</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>LifecycleController</x:v>
+        <x:v>DC-03 LifecycleController</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
         <x:v>부분 Open Rollback과 데이터 보존 시험</x:v>
@@ -969,7 +972,7 @@
         <x:v>FR-LIFE-025~032; ERR-037~038</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="32" customHeight="1">
+    <x:row r="9" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A9" s="22" t="str">
         <x:v>REQ-FUNC-008</x:v>
       </x:c>
@@ -980,7 +983,7 @@
         <x:v>FS-SHUT-001</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
-        <x:v>EmulatorContext; LifecycleController</x:v>
+        <x:v>DC-02 EmulatorContext; DC-03 LifecycleController</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>각 상태 Finalize, Cancel I/O, 재초기화 시험</x:v>
@@ -993,7 +996,7 @@
         <x:v>FR-LIFE-017~022</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="32" customHeight="1">
+    <x:row r="10" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A10" s="22" t="str">
         <x:v>REQ-FUNC-009</x:v>
       </x:c>
@@ -1004,7 +1007,7 @@
         <x:v>FS-CSV-001</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>CAPL Core; ConfigurationLoader</x:v>
+        <x:v>DC-04 ConfigurationLoader; DC-13 CAPL Core</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
         <x:v>프로젝트 이동·파일명 변경·경로 변환 실패 시험</x:v>
@@ -1017,7 +1020,7 @@
         <x:v>FR-CSV-001~003; DATA-001~002</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="32" customHeight="1">
+    <x:row r="11" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A11" s="22" t="str">
         <x:v>REQ-FUNC-010</x:v>
       </x:c>
@@ -1028,7 +1031,7 @@
         <x:v>FS-CSV-001</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
-        <x:v>ConfigurationLoader</x:v>
+        <x:v>DC-04 ConfigurationLoader</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
         <x:v>다수 CSV 혼재 환경의 정확한 파일 선택 시험</x:v>
@@ -1041,7 +1044,7 @@
         <x:v>FR-CSV-001~003; IF-CORE-009</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="32" customHeight="1">
+    <x:row r="12" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A12" s="22" t="str">
         <x:v>REQ-FUNC-011</x:v>
       </x:c>
@@ -1052,7 +1055,7 @@
         <x:v>FS-CSV-002,FS-CSV-003</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
-        <x:v>ConfigurationLoader; LifecycleController</x:v>
+        <x:v>DC-03 LifecycleController; DC-04 ConfigurationLoader</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
         <x:v>성공/실패 원자성 및 Connected 거부 시험</x:v>
@@ -1065,7 +1068,7 @@
         <x:v>FR-CSV-004~010,014~019</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="32" customHeight="1">
+    <x:row r="13" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A13" s="22" t="str">
         <x:v>REQ-FUNC-012</x:v>
       </x:c>
@@ -1076,7 +1079,7 @@
         <x:v>FS-CSV-003</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
-        <x:v>ConfigurationLoader; SnapshotService; DiagnosticService</x:v>
+        <x:v>DC-04 ConfigurationLoader; DC-11 SnapshotService; DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E13" s="9" t="str">
         <x:v>Refresh 전후 값과 런타임 상태 초기화 시험</x:v>
@@ -1089,7 +1092,7 @@
         <x:v>FR-CSV-005,012,017~019</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="32" customHeight="1">
+    <x:row r="14" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A14" s="22" t="str">
         <x:v>REQ-FUNC-013</x:v>
       </x:c>
@@ -1100,7 +1103,7 @@
         <x:v>FS-CSV-003</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str">
-        <x:v>ConfigurationLoader; LifecycleController</x:v>
+        <x:v>DC-03 LifecycleController; DC-04 ConfigurationLoader</x:v>
       </x:c>
       <x:c r="E14" s="9" t="str">
         <x:v>Stale Configuration 차단 및 재시도 시험</x:v>
@@ -1113,7 +1116,7 @@
         <x:v>FR-CSV-006~008,015~016; ERR-035~036</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="32" customHeight="1">
+    <x:row r="15" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A15" s="22" t="str">
         <x:v>REQ-FUNC-014</x:v>
       </x:c>
@@ -1124,7 +1127,7 @@
         <x:v>FS-DEV-001</x:v>
       </x:c>
       <x:c r="D15" s="9" t="str">
-        <x:v>DeviceRegistry</x:v>
+        <x:v>DC-05 DeviceRegistry</x:v>
       </x:c>
       <x:c r="E15" s="9" t="str">
         <x:v>동일 Port 다중 Slave와 다른 Port 동일 Slave ID 시험</x:v>
@@ -1137,7 +1140,7 @@
         <x:v>FR-RTU-007; DATA-DEV-001~006</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="32" customHeight="1">
+    <x:row r="16" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A16" s="22" t="str">
         <x:v>REQ-FUNC-015</x:v>
       </x:c>
@@ -1148,7 +1151,7 @@
         <x:v>FS-REG-001</x:v>
       </x:c>
       <x:c r="D16" s="9" t="str">
-        <x:v>RegisterService; DeviceRegistry</x:v>
+        <x:v>DC-05 DeviceRegistry; DC-06 RegisterService</x:v>
       </x:c>
       <x:c r="E16" s="9" t="str">
         <x:v>동일 Address의 FC03/FC04 동일값 시험</x:v>
@@ -1161,7 +1164,7 @@
         <x:v>FR-REG-001~009</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="32" customHeight="1">
+    <x:row r="17" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A17" s="22" t="str">
         <x:v>REQ-FUNC-016</x:v>
       </x:c>
@@ -1172,7 +1175,7 @@
         <x:v>FS-REG-001,FS-REG-002</x:v>
       </x:c>
       <x:c r="D17" s="9" t="str">
-        <x:v>RegisterService</x:v>
+        <x:v>DC-06 RegisterService</x:v>
       </x:c>
       <x:c r="E17" s="9" t="str">
         <x:v>Rule-only, Map-only, 공백 범위 접근 시험</x:v>
@@ -1185,7 +1188,7 @@
         <x:v>FR-REG-013~017; DATA-020,024</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="32" customHeight="1">
+    <x:row r="18" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A18" s="22" t="str">
         <x:v>REQ-FUNC-017</x:v>
       </x:c>
@@ -1196,7 +1199,7 @@
         <x:v>FS-REG-001,FS-REG-002</x:v>
       </x:c>
       <x:c r="D18" s="9" t="str">
-        <x:v>RegisterService</x:v>
+        <x:v>DC-06 RegisterService</x:v>
       </x:c>
       <x:c r="E18" s="9" t="str">
         <x:v>경계·Buffer 부족·동시 접근 원자성 시험</x:v>
@@ -1209,7 +1212,7 @@
         <x:v>FR-REG-015~018; IF-REG-001~012</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="32" customHeight="1">
+    <x:row r="19" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A19" s="22" t="str">
         <x:v>REQ-FUNC-018</x:v>
       </x:c>
@@ -1220,7 +1223,7 @@
         <x:v>FS-REG-002,FS-MON-004</x:v>
       </x:c>
       <x:c r="D19" s="9" t="str">
-        <x:v>RegisterService; SnapshotService</x:v>
+        <x:v>DC-06 RegisterService; DC-11 SnapshotService</x:v>
       </x:c>
       <x:c r="E19" s="9" t="str">
         <x:v>중첩 Rule, 동일값 Write 및 중복 제거 시험</x:v>
@@ -1233,7 +1236,7 @@
         <x:v>FR-REG-010~012,018</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="32" customHeight="1">
+    <x:row r="20" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A20" s="22" t="str">
         <x:v>REQ-FUNC-019</x:v>
       </x:c>
@@ -1244,7 +1247,7 @@
         <x:v>FS-REG-003</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
-        <x:v>RegisterService; SnapshotService</x:v>
+        <x:v>DC-06 RegisterService; DC-11 SnapshotService</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
         <x:v>Connected/Disconnected Reset과 실패 Rollback 시험</x:v>
@@ -1257,7 +1260,7 @@
         <x:v>FR-RESET-001~007</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="32" customHeight="1">
+    <x:row r="21" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A21" s="22" t="str">
         <x:v>REQ-FUNC-020</x:v>
       </x:c>
@@ -1268,7 +1271,7 @@
         <x:v>FS-SIG-001,FS-SIG-002,FS-SIG-003</x:v>
       </x:c>
       <x:c r="D21" s="9" t="str">
-        <x:v>SignalCodec</x:v>
+        <x:v>DC-07 SignalCodec</x:v>
       </x:c>
       <x:c r="E21" s="9" t="str">
         <x:v>SignalName 대소문자·중복·미존재 시험</x:v>
@@ -1281,7 +1284,7 @@
         <x:v>FR-SIG-001~006; DATA-MAP-023</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="32" customHeight="1">
+    <x:row r="22" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A22" s="22" t="str">
         <x:v>REQ-FUNC-021</x:v>
       </x:c>
@@ -1292,7 +1295,7 @@
         <x:v>FS-SIG-002,FS-SIG-003,FS-SIG-004</x:v>
       </x:c>
       <x:c r="D22" s="9" t="str">
-        <x:v>SignalCodec</x:v>
+        <x:v>DC-07 SignalCodec</x:v>
       </x:c>
       <x:c r="E22" s="9" t="str">
         <x:v>양·음수 Scale/Offset 및 ±0.5 반올림 시험</x:v>
@@ -1305,7 +1308,7 @@
         <x:v>FR-SIG-025~030</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="32" customHeight="1">
+    <x:row r="23" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A23" s="22" t="str">
         <x:v>REQ-FUNC-022</x:v>
       </x:c>
@@ -1316,7 +1319,7 @@
         <x:v>FS-SIG-002,FS-SIG-003,FS-SIG-004</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str">
-        <x:v>SignalCodec</x:v>
+        <x:v>DC-07 SignalCodec</x:v>
       </x:c>
       <x:c r="E23" s="9" t="str">
         <x:v>Float/Double Raw round-trip 및 비유한 값 시험</x:v>
@@ -1329,7 +1332,7 @@
         <x:v>FR-SIG-007~008; DATA-MAP-008~009</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="32" customHeight="1">
+    <x:row r="24" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A24" s="22" t="str">
         <x:v>REQ-FUNC-023</x:v>
       </x:c>
@@ -1340,7 +1343,7 @@
         <x:v>FS-SIG-001~004</x:v>
       </x:c>
       <x:c r="D24" s="9" t="str">
-        <x:v>SignalCodec</x:v>
+        <x:v>DC-07 SignalCodec</x:v>
       </x:c>
       <x:c r="E24" s="9" t="str">
         <x:v>2/4 Word Address별 Raw 배치 시험</x:v>
@@ -1353,7 +1356,7 @@
         <x:v>FR-SIG-009~010; DATA-MAP-010</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="32" customHeight="1">
+    <x:row r="25" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A25" s="22" t="str">
         <x:v>REQ-FUNC-024</x:v>
       </x:c>
@@ -1364,7 +1367,7 @@
         <x:v>FS-SIG-001~004</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
-        <x:v>SignalCodec</x:v>
+        <x:v>DC-07 SignalCodec</x:v>
       </x:c>
       <x:c r="E25" s="9" t="str">
         <x:v>Length 2/4/6/8의 Bit 경계·비정렬 Signal 시험</x:v>
@@ -1377,7 +1380,7 @@
         <x:v>FR-SIG-011~014</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="32" customHeight="1">
+    <x:row r="26" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A26" s="22" t="str">
         <x:v>REQ-FUNC-025</x:v>
       </x:c>
@@ -1388,7 +1391,7 @@
         <x:v>FS-SIG-001~004</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
-        <x:v>SignalCodec</x:v>
+        <x:v>DC-07 SignalCodec</x:v>
       </x:c>
       <x:c r="E26" s="9" t="str">
         <x:v>Big/Little Endian Read/Write 역변환 시험</x:v>
@@ -1401,7 +1404,7 @@
         <x:v>FR-SIG-020~024</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="32" customHeight="1">
+    <x:row r="27" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A27" s="22" t="str">
         <x:v>REQ-FUNC-026</x:v>
       </x:c>
@@ -1412,7 +1415,7 @@
         <x:v>FS-CSV-002,FS-SIG-001</x:v>
       </x:c>
       <x:c r="D27" s="9" t="str">
-        <x:v>ConfigurationLoader; SignalCodec</x:v>
+        <x:v>DC-04 ConfigurationLoader; DC-07 SignalCodec</x:v>
       </x:c>
       <x:c r="E27" s="9" t="str">
         <x:v>Frame 공유·중복·경계 검증 시험</x:v>
@@ -1425,7 +1428,7 @@
         <x:v>FR-SIG-012,015~019; DATA-MAP-011~014</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="32" customHeight="1">
+    <x:row r="28" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A28" s="22" t="str">
         <x:v>REQ-FUNC-027</x:v>
       </x:c>
@@ -1436,7 +1439,7 @@
         <x:v>FS-SIG-004</x:v>
       </x:c>
       <x:c r="D28" s="9" t="str">
-        <x:v>ConfigurationLoader; SignalCodec</x:v>
+        <x:v>DC-04 ConfigurationLoader; DC-07 SignalCodec</x:v>
       </x:c>
       <x:c r="E28" s="9" t="str">
         <x:v>행 순서 변경·부분 실패 Rollback 시험</x:v>
@@ -1449,7 +1452,7 @@
         <x:v>FR-SIG-025~027; DATA-MAP-004</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="32" customHeight="1">
+    <x:row r="29" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A29" s="22" t="str">
         <x:v>REQ-FUNC-028</x:v>
       </x:c>
@@ -1460,7 +1463,7 @@
         <x:v>FS-SIG-002~004</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str">
-        <x:v>SignalCodec; RegisterService</x:v>
+        <x:v>DC-06 RegisterService; DC-07 SignalCodec</x:v>
       </x:c>
       <x:c r="E29" s="9" t="str">
         <x:v>Min/Max 경계, Raw 우회 및 NaN/Infinity 시험</x:v>
@@ -1473,7 +1476,7 @@
         <x:v>FR-SIG-031~037</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="32" customHeight="1">
+    <x:row r="30" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A30" s="22" t="str">
         <x:v>REQ-FUNC-029</x:v>
       </x:c>
@@ -1484,7 +1487,7 @@
         <x:v>FS-SIG-002,FS-SIG-003</x:v>
       </x:c>
       <x:c r="D30" s="9" t="str">
-        <x:v>CAPL ABI Adapter; SignalCodec</x:v>
+        <x:v>DC-01 CAPL ABI Adapter; DC-07 SignalCodec</x:v>
       </x:c>
       <x:c r="E30" s="9" t="str">
         <x:v>±2^53 경계 및 word[4] Raw 우회 시험</x:v>
@@ -1497,7 +1500,7 @@
         <x:v>FR-SIG-038~041; IF-SIG-006~007</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="32" customHeight="1">
+    <x:row r="31" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A31" s="22" t="str">
         <x:v>REQ-FUNC-030</x:v>
       </x:c>
@@ -1508,7 +1511,7 @@
         <x:v>FS-MON-001</x:v>
       </x:c>
       <x:c r="D31" s="9" t="str">
-        <x:v>CAPL UI; SnapshotService</x:v>
+        <x:v>DC-11 SnapshotService; DC-15 CAPL UI</x:v>
       </x:c>
       <x:c r="E31" s="9" t="str">
         <x:v>ON/OFF 중 RTU 유지와 Queue 정책 시험</x:v>
@@ -1521,7 +1524,7 @@
         <x:v>FR-LIFE-004~006; FR-CAN-049~056</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="32" customHeight="1">
+    <x:row r="32" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A32" s="22" t="str">
         <x:v>REQ-FUNC-031</x:v>
       </x:c>
@@ -1532,7 +1535,7 @@
         <x:v>FS-MON-002</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str">
-        <x:v>CAPL Monitoring</x:v>
+        <x:v>DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E32" s="9" t="str">
         <x:v>다중 Checkbox 원자 적용·복원 시험</x:v>
@@ -1545,7 +1548,7 @@
         <x:v>FR-CAN-020~027,047,057</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="32" customHeight="1">
+    <x:row r="33" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A33" s="22" t="str">
         <x:v>REQ-FUNC-032</x:v>
       </x:c>
@@ -1556,7 +1559,7 @@
         <x:v>FS-MON-001,FS-MON-003</x:v>
       </x:c>
       <x:c r="D33" s="9" t="str">
-        <x:v>CAPL Monitoring; SnapshotService</x:v>
+        <x:v>DC-11 SnapshotService; DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E33" s="9" t="str">
         <x:v>Connect/ReadSwitch 순서 및 최초 출력 시험</x:v>
@@ -1569,7 +1572,7 @@
         <x:v>FR-LIFE-007~008; FR-CAN-055</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="32" customHeight="1">
+    <x:row r="34" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A34" s="22" t="str">
         <x:v>REQ-FUNC-033</x:v>
       </x:c>
@@ -1580,7 +1583,7 @@
         <x:v>FS-MON-003,FS-MON-006</x:v>
       </x:c>
       <x:c r="D34" s="9" t="str">
-        <x:v>CAPL Monitoring</x:v>
+        <x:v>DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E34" s="9" t="str">
         <x:v>Deadline Miss·Latest-wins·공정성 시험</x:v>
@@ -1593,7 +1596,7 @@
         <x:v>FR-CAN-022,042~048; FR-LOAD-007</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="32" customHeight="1">
+    <x:row r="35" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A35" s="22" t="str">
         <x:v>REQ-FUNC-034</x:v>
       </x:c>
@@ -1604,7 +1607,7 @@
         <x:v>FS-MON-004</x:v>
       </x:c>
       <x:c r="D35" s="9" t="str">
-        <x:v>SnapshotService; CAPL Monitoring</x:v>
+        <x:v>DC-11 SnapshotService; DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E35" s="9" t="str">
         <x:v>동시 Write·불변 Snapshot·Buffer 부족 시험</x:v>
@@ -1617,7 +1620,7 @@
         <x:v>FR-CAN-029~037; IF-MON-006~010</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="32" customHeight="1">
+    <x:row r="36" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A36" s="22" t="str">
         <x:v>REQ-FUNC-035</x:v>
       </x:c>
@@ -1628,7 +1631,7 @@
         <x:v>FS-MON-004,FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D36" s="9" t="str">
-        <x:v>SnapshotService; DiagnosticService</x:v>
+        <x:v>DC-11 SnapshotService; DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E36" s="9" t="str">
         <x:v>Queue 257건 입력 및 oldest-drop 시험</x:v>
@@ -1641,7 +1644,7 @@
         <x:v>FR-CAN-038~039; ERR-008; FR-LOAD-008</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="32" customHeight="1">
+    <x:row r="37" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A37" s="22" t="str">
         <x:v>REQ-FUNC-036</x:v>
       </x:c>
@@ -1652,7 +1655,7 @@
         <x:v>FS-MON-006</x:v>
       </x:c>
       <x:c r="D37" s="9" t="str">
-        <x:v>CAPL Monitoring</x:v>
+        <x:v>DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E37" s="9" t="str">
         <x:v>두 Port Burst·Rule Cursor·묶음 원자 출력 시험</x:v>
@@ -1665,7 +1668,7 @@
         <x:v>FR-CAN-040~046; DES-CAN-014~017</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="32" customHeight="1">
+    <x:row r="38" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A38" s="22" t="str">
         <x:v>REQ-FUNC-037</x:v>
       </x:c>
@@ -1676,7 +1679,7 @@
         <x:v>FS-MON-006</x:v>
       </x:c>
       <x:c r="D38" s="9" t="str">
-        <x:v>CAPL Monitoring</x:v>
+        <x:v>DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E38" s="9" t="str">
         <x:v>Quantity 125 Snapshot과 Tick 시간 실측</x:v>
@@ -1689,7 +1692,7 @@
         <x:v>FR-LOAD-006,019</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="32" customHeight="1">
+    <x:row r="39" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A39" s="22" t="str">
         <x:v>REQ-FUNC-038</x:v>
       </x:c>
@@ -1700,7 +1703,7 @@
         <x:v>FS-MON-002,FS-MON-006</x:v>
       </x:c>
       <x:c r="D39" s="9" t="str">
-        <x:v>CAPL Monitoring; DiagnosticService</x:v>
+        <x:v>DC-12 DiagnosticService; DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E39" s="9" t="str">
         <x:v>Performance Monitor 유무·임의값 불변 동작 시험</x:v>
@@ -1713,7 +1716,7 @@
         <x:v>FR-LOAD-001~005,010,018</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="32" customHeight="1">
+    <x:row r="40" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A40" s="22" t="str">
         <x:v>REQ-FUNC-039</x:v>
       </x:c>
@@ -1724,7 +1727,7 @@
         <x:v>FS-MON-001,FS-MON-004</x:v>
       </x:c>
       <x:c r="D40" s="9" t="str">
-        <x:v>SnapshotService</x:v>
+        <x:v>DC-11 SnapshotService</x:v>
       </x:c>
       <x:c r="E40" s="9" t="str">
         <x:v>OFF 전후 Queue·Counter·재시작 Burst 시험</x:v>
@@ -1737,7 +1740,7 @@
         <x:v>FR-CAN-051~056; FR-LOAD-015~018</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="32" customHeight="1">
+    <x:row r="41" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A41" s="22" t="str">
         <x:v>REQ-FUNC-040</x:v>
       </x:c>
@@ -1748,7 +1751,7 @@
         <x:v>FS-UI-001,FS-UI-002,FS-UI-003</x:v>
       </x:c>
       <x:c r="D41" s="9" t="str">
-        <x:v>CAPL Core; CAPL Monitoring; CAPL UI</x:v>
+        <x:v>DC-13 CAPL Core; DC-14 CAPL Monitoring; DC-15 CAPL UI</x:v>
       </x:c>
       <x:c r="E41" s="9" t="str">
         <x:v>CAPL 정적 분석 및 컴파일 시험</x:v>
@@ -1761,7 +1764,7 @@
         <x:v>FR-CAPL-001~006; IF-CTX-006</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="32" customHeight="1">
+    <x:row r="42" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A42" s="22" t="str">
         <x:v>REQ-FUNC-041</x:v>
       </x:c>
@@ -1772,7 +1775,7 @@
         <x:v>FS-UI-001</x:v>
       </x:c>
       <x:c r="D42" s="9" t="str">
-        <x:v>CAPL UI; RegisterService</x:v>
+        <x:v>DC-06 RegisterService; DC-15 CAPL UI</x:v>
       </x:c>
       <x:c r="E42" s="9" t="str">
         <x:v>Panel 수동 Read 및 실패 시 결과 유지 시험</x:v>
@@ -1785,7 +1788,7 @@
         <x:v>FR-UI-001~006; IF-REG-001,004</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="32" customHeight="1">
+    <x:row r="43" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A43" s="22" t="str">
         <x:v>REQ-FUNC-042</x:v>
       </x:c>
@@ -1796,7 +1799,7 @@
         <x:v>FS-UI-002</x:v>
       </x:c>
       <x:c r="D43" s="9" t="str">
-        <x:v>CAPL UI; RegisterService</x:v>
+        <x:v>DC-06 RegisterService; DC-15 CAPL UI</x:v>
       </x:c>
       <x:c r="E43" s="9" t="str">
         <x:v>Panel 편집 중간 상태와 실행 Snapshot 분리 시험</x:v>
@@ -1809,7 +1812,7 @@
         <x:v>FR-UI-007~011; IF-REG-002~016</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" ht="32" customHeight="1">
+    <x:row r="44" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A44" s="22" t="str">
         <x:v>REQ-FUNC-043</x:v>
       </x:c>
@@ -1820,7 +1823,7 @@
         <x:v>FS-UI-001</x:v>
       </x:c>
       <x:c r="D44" s="9" t="str">
-        <x:v>CAPL UI</x:v>
+        <x:v>DC-15 CAPL UI</x:v>
       </x:c>
       <x:c r="E44" s="9" t="str">
         <x:v>Auto Read, Send momentary 및 invalid edit 시험</x:v>
@@ -1833,7 +1836,7 @@
         <x:v>FR-UI-012~016</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="32" customHeight="1">
+    <x:row r="45" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A45" s="22" t="str">
         <x:v>REQ-FUNC-044</x:v>
       </x:c>
@@ -1844,7 +1847,7 @@
         <x:v>FS-UI-003</x:v>
       </x:c>
       <x:c r="D45" s="9" t="str">
-        <x:v>CAPL UI; SignalCodec</x:v>
+        <x:v>DC-07 SignalCodec; DC-15 CAPL UI</x:v>
       </x:c>
       <x:c r="E45" s="9" t="str">
         <x:v>양수·음수·소수 Panel round-trip 시험</x:v>
@@ -1857,7 +1860,7 @@
         <x:v>FR-SIG-003; IF-SIG-001~007</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="32" customHeight="1">
+    <x:row r="46" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A46" s="22" t="str">
         <x:v>REQ-COM-001</x:v>
       </x:c>
@@ -1868,7 +1871,7 @@
         <x:v>FS-COM-001</x:v>
       </x:c>
       <x:c r="D46" s="9" t="str">
-        <x:v>Win32SerialPort</x:v>
+        <x:v>DC-09 Win32SerialPort</x:v>
       </x:c>
       <x:c r="E46" s="9" t="str">
         <x:v>회사 환경 SystemBase Multi USB-485 통합 시험</x:v>
@@ -1881,7 +1884,7 @@
         <x:v>ENV-003,014~015; CON-017</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="32" customHeight="1">
+    <x:row r="47" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A47" s="22" t="str">
         <x:v>REQ-COM-002</x:v>
       </x:c>
@@ -1892,7 +1895,7 @@
         <x:v>FS-COM-001</x:v>
       </x:c>
       <x:c r="D47" s="9" t="str">
-        <x:v>DeviceRegistry; CAPL Core</x:v>
+        <x:v>DC-05 DeviceRegistry; DC-13 CAPL Core</x:v>
       </x:c>
       <x:c r="E47" s="9" t="str">
         <x:v>Port 등록 순서·중복·누락·Routing 시험</x:v>
@@ -1905,7 +1908,7 @@
         <x:v>ENV-003~005; FR-PORT-018~020</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="32" customHeight="1">
+    <x:row r="48" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A48" s="22" t="str">
         <x:v>REQ-COM-003</x:v>
       </x:c>
@@ -1916,7 +1919,7 @@
         <x:v>FS-COM-001</x:v>
       </x:c>
       <x:c r="D48" s="9" t="str">
-        <x:v>Win32SerialPort</x:v>
+        <x:v>DC-09 Win32SerialPort</x:v>
       </x:c>
       <x:c r="E48" s="9" t="str">
         <x:v>지원/비지원 설정 및 상태 제한 시험</x:v>
@@ -1929,7 +1932,7 @@
         <x:v>FR-PORT-001~006</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="32" customHeight="1">
+    <x:row r="49" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A49" s="22" t="str">
         <x:v>REQ-COM-004</x:v>
       </x:c>
@@ -1940,7 +1943,7 @@
         <x:v>FS-COM-001</x:v>
       </x:c>
       <x:c r="D49" s="9" t="str">
-        <x:v>Win32SerialPort</x:v>
+        <x:v>DC-09 Win32SerialPort</x:v>
       </x:c>
       <x:c r="E49" s="9" t="str">
         <x:v>BaudRate·Parity·StopBits 조합과 OS 오류 Context 시험</x:v>
@@ -1953,7 +1956,7 @@
         <x:v>FR-PORT-002,010~012</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="32" customHeight="1">
+    <x:row r="50" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A50" s="22" t="str">
         <x:v>REQ-COM-005</x:v>
       </x:c>
@@ -1964,7 +1967,7 @@
         <x:v>FS-COM-001</x:v>
       </x:c>
       <x:c r="D50" s="9" t="str">
-        <x:v>Win32SerialPort</x:v>
+        <x:v>DC-09 Win32SerialPort</x:v>
       </x:c>
       <x:c r="E50" s="9" t="str">
         <x:v>RTS 미조작 및 Echo 없는 Adapter 확인</x:v>
@@ -1977,7 +1980,7 @@
         <x:v>FR-PORT-022~023</x:v>
       </x:c>
     </x:row>
-    <x:row r="51" ht="32" customHeight="1">
+    <x:row r="51" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A51" s="22" t="str">
         <x:v>REQ-COM-006</x:v>
       </x:c>
@@ -1988,7 +1991,7 @@
         <x:v>FS-MODBUS-002~005</x:v>
       </x:c>
       <x:c r="D51" s="9" t="str">
-        <x:v>ModbusRtuEngine</x:v>
+        <x:v>DC-08 ModbusRtuEngine</x:v>
       </x:c>
       <x:c r="E51" s="9" t="str">
         <x:v>Function별 정상·미지원 요청 시험</x:v>
@@ -2001,7 +2004,7 @@
         <x:v>FR-RTU-001~006,015~016</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="32" customHeight="1">
+    <x:row r="52" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A52" s="22" t="str">
         <x:v>REQ-COM-007</x:v>
       </x:c>
@@ -2012,7 +2015,7 @@
         <x:v>FS-MODBUS-002~005</x:v>
       </x:c>
       <x:c r="D52" s="9" t="str">
-        <x:v>ModbusRtuEngine</x:v>
+        <x:v>DC-08 ModbusRtuEngine</x:v>
       </x:c>
       <x:c r="E52" s="9" t="str">
         <x:v>최소·최대·초과 및 ByteCount 오류 시험</x:v>
@@ -2025,7 +2028,7 @@
         <x:v>FR-RTU-017~020,028~031</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" ht="32" customHeight="1">
+    <x:row r="53" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A53" s="22" t="str">
         <x:v>REQ-COM-008</x:v>
       </x:c>
@@ -2036,7 +2039,7 @@
         <x:v>FS-MODBUS-002~004</x:v>
       </x:c>
       <x:c r="D53" s="9" t="str">
-        <x:v>ModbusRtuEngine; RegisterService</x:v>
+        <x:v>DC-06 RegisterService; DC-08 ModbusRtuEngine</x:v>
       </x:c>
       <x:c r="E53" s="9" t="str">
         <x:v>인접·중첩 Rule 횡단과 공백 거부 시험</x:v>
@@ -2049,7 +2052,7 @@
         <x:v>FR-RTU-010~014; DATA-RULE-012</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="32" customHeight="1">
+    <x:row r="54" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A54" s="22" t="str">
         <x:v>REQ-COM-009</x:v>
       </x:c>
@@ -2060,7 +2063,7 @@
         <x:v>FS-MODBUS-004</x:v>
       </x:c>
       <x:c r="D54" s="9" t="str">
-        <x:v>ModbusRtuEngine; RegisterService</x:v>
+        <x:v>DC-06 RegisterService; DC-08 ModbusRtuEngine</x:v>
       </x:c>
       <x:c r="E54" s="9" t="str">
         <x:v>적용 전/후 송신 실패 Stage 시험</x:v>
@@ -2073,7 +2076,7 @@
         <x:v>FR-RTU-031~032; ERR-043</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="32" customHeight="1">
+    <x:row r="55" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A55" s="22" t="str">
         <x:v>REQ-COM-010</x:v>
       </x:c>
@@ -2084,7 +2087,7 @@
         <x:v>FS-MODBUS-001,FS-MODBUS-005</x:v>
       </x:c>
       <x:c r="D55" s="9" t="str">
-        <x:v>DeviceRegistry; ModbusRtuEngine</x:v>
+        <x:v>DC-05 DeviceRegistry; DC-08 ModbusRtuEngine</x:v>
       </x:c>
       <x:c r="E55" s="9" t="str">
         <x:v>Broadcast·예약·미등록 주소 시험</x:v>
@@ -2097,7 +2100,7 @@
         <x:v>FR-RTU-021~022</x:v>
       </x:c>
     </x:row>
-    <x:row r="56" ht="32" customHeight="1">
+    <x:row r="56" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A56" s="22" t="str">
         <x:v>REQ-COM-011</x:v>
       </x:c>
@@ -2108,7 +2111,7 @@
         <x:v>FS-COM-003</x:v>
       </x:c>
       <x:c r="D56" s="9" t="str">
-        <x:v>ModbusRtuEngine</x:v>
+        <x:v>DC-08 ModbusRtuEngine</x:v>
       </x:c>
       <x:c r="E56" s="9" t="str">
         <x:v>공식 CRC Vector·최대 ADU 시험</x:v>
@@ -2121,7 +2124,7 @@
         <x:v>FR-RTU-023,026~030</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="32" customHeight="1">
+    <x:row r="57" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A57" s="22" t="str">
         <x:v>REQ-COM-012</x:v>
       </x:c>
@@ -2132,7 +2135,7 @@
         <x:v>FS-COM-002</x:v>
       </x:c>
       <x:c r="D57" s="9" t="str">
-        <x:v>PortWorker; Win32SerialPort</x:v>
+        <x:v>DC-09 Win32SerialPort; DC-10 PortWorker</x:v>
       </x:c>
       <x:c r="E57" s="9" t="str">
         <x:v>Partial Read, Noise, t1.5/t3.5 경계 시험</x:v>
@@ -2145,7 +2148,7 @@
         <x:v>FR-RTU-024~025,035; FR-PORT-021</x:v>
       </x:c>
     </x:row>
-    <x:row r="58" ht="32" customHeight="1">
+    <x:row r="58" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A58" s="22" t="str">
         <x:v>REQ-COM-013</x:v>
       </x:c>
@@ -2156,7 +2159,7 @@
         <x:v>FS-COM-002</x:v>
       </x:c>
       <x:c r="D58" s="9" t="str">
-        <x:v>PortWorker</x:v>
+        <x:v>DC-10 PortWorker</x:v>
       </x:c>
       <x:c r="E58" s="9" t="str">
         <x:v>다양한 BaudRate/Parity/StopBits Timing 시험</x:v>
@@ -2169,7 +2172,7 @@
         <x:v>FR-RTU-025; FR-PORT-021</x:v>
       </x:c>
     </x:row>
-    <x:row r="59" ht="32" customHeight="1">
+    <x:row r="59" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A59" s="22" t="str">
         <x:v>REQ-COM-014</x:v>
       </x:c>
@@ -2180,7 +2183,7 @@
         <x:v>FS-COM-003,FS-MODBUS-005</x:v>
       </x:c>
       <x:c r="D59" s="9" t="str">
-        <x:v>ModbusRtuEngine; DiagnosticService</x:v>
+        <x:v>DC-08 ModbusRtuEngine; DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E59" s="9" t="str">
         <x:v>Noise 반복 시 FIFO 고갈 방지 시험</x:v>
@@ -2193,7 +2196,7 @@
         <x:v>FR-RTU-027; ERR-040</x:v>
       </x:c>
     </x:row>
-    <x:row r="60" ht="32" customHeight="1">
+    <x:row r="60" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A60" s="22" t="str">
         <x:v>REQ-COM-015</x:v>
       </x:c>
@@ -2204,7 +2207,7 @@
         <x:v>FS-MODBUS-001</x:v>
       </x:c>
       <x:c r="D60" s="9" t="str">
-        <x:v>PortWorker</x:v>
+        <x:v>DC-10 PortWorker</x:v>
       </x:c>
       <x:c r="E60" s="9" t="str">
         <x:v>두 Port 동시 요청·순서·격리 시험</x:v>
@@ -2217,7 +2220,7 @@
         <x:v>FR-RTU-034</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="32" customHeight="1">
+    <x:row r="61" ht="15" hidden="0" customHeight="1">
       <x:c r="A61" s="22" t="str">
         <x:v>REQ-COM-016</x:v>
       </x:c>
@@ -2228,7 +2231,7 @@
         <x:v>FS-MON-005</x:v>
       </x:c>
       <x:c r="D61" s="9" t="str">
-        <x:v>CAPL Monitoring</x:v>
+        <x:v>DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E61" s="9" t="str">
         <x:v>두 가상 채널 Extended CAN 출력 시험</x:v>
@@ -2241,7 +2244,7 @@
         <x:v>ENV-007,012</x:v>
       </x:c>
     </x:row>
-    <x:row r="62" ht="32" customHeight="1">
+    <x:row r="62" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A62" s="22" t="str">
         <x:v>REQ-COM-017</x:v>
       </x:c>
@@ -2252,7 +2255,7 @@
         <x:v>FS-MON-005</x:v>
       </x:c>
       <x:c r="D62" s="9" t="str">
-        <x:v>CAPL Monitoring</x:v>
+        <x:v>DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E62" s="9" t="str">
         <x:v>실제 ID/Vector 표현 Mask 시험</x:v>
@@ -2265,7 +2268,7 @@
         <x:v>FR-CAN-001~002,021; CON-001</x:v>
       </x:c>
     </x:row>
-    <x:row r="63" ht="32" customHeight="1">
+    <x:row r="63" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A63" s="22" t="str">
         <x:v>REQ-COM-018</x:v>
       </x:c>
@@ -2276,7 +2279,7 @@
         <x:v>FS-MON-005</x:v>
       </x:c>
       <x:c r="D63" s="9" t="str">
-        <x:v>CAPL Monitoring</x:v>
+        <x:v>DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E63" s="9" t="str">
         <x:v>Quantity 1,4,5,125 Frame 수·mm 시험</x:v>
@@ -2289,7 +2292,7 @@
         <x:v>FR-CAN-003~019,028</x:v>
       </x:c>
     </x:row>
-    <x:row r="64" ht="32" customHeight="1">
+    <x:row r="64" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A64" s="22" t="str">
         <x:v>REQ-COM-019</x:v>
       </x:c>
@@ -2300,7 +2303,7 @@
         <x:v>FS-MON-005</x:v>
       </x:c>
       <x:c r="D64" s="9" t="str">
-        <x:v>CAPL Monitoring</x:v>
+        <x:v>DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E64" s="9" t="str">
         <x:v>Header Byte 단위 Golden Vector 시험</x:v>
@@ -2313,7 +2316,7 @@
         <x:v>FR-CAN-003~012</x:v>
       </x:c>
     </x:row>
-    <x:row r="65" ht="32" customHeight="1">
+    <x:row r="65" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A65" s="22" t="str">
         <x:v>REQ-COM-020</x:v>
       </x:c>
@@ -2324,7 +2327,7 @@
         <x:v>FS-MON-005</x:v>
       </x:c>
       <x:c r="D65" s="9" t="str">
-        <x:v>CAPL Monitoring</x:v>
+        <x:v>DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E65" s="9" t="str">
         <x:v>마지막 가변 DLC 및 무패딩 시험</x:v>
@@ -2337,7 +2340,7 @@
         <x:v>FR-CAN-013~019</x:v>
       </x:c>
     </x:row>
-    <x:row r="66" ht="32" customHeight="1">
+    <x:row r="66" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A66" s="22" t="str">
         <x:v>REQ-COM-021</x:v>
       </x:c>
@@ -2348,7 +2351,7 @@
         <x:v>FS-MON-003~005</x:v>
       </x:c>
       <x:c r="D66" s="9" t="str">
-        <x:v>SnapshotService</x:v>
+        <x:v>DC-11 SnapshotService</x:v>
       </x:c>
       <x:c r="E66" s="9" t="str">
         <x:v>원인별 Header 및 0x04 미송출 시험</x:v>
@@ -2361,7 +2364,7 @@
         <x:v>FR-SRC-001~005; FR-LIFE-008</x:v>
       </x:c>
     </x:row>
-    <x:row r="67" ht="32" customHeight="1">
+    <x:row r="67" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A67" s="22" t="str">
         <x:v>REQ-DATA-001</x:v>
       </x:c>
@@ -2372,7 +2375,7 @@
         <x:v>FS-CSV-002,FS-MODBUS-002~004</x:v>
       </x:c>
       <x:c r="D67" s="9" t="str">
-        <x:v>ConfigurationLoader; RegisterService</x:v>
+        <x:v>DC-04 ConfigurationLoader; DC-06 RegisterService</x:v>
       </x:c>
       <x:c r="E67" s="9" t="str">
         <x:v>Address 0,40000,65535 경계 시험</x:v>
@@ -2385,7 +2388,7 @@
         <x:v>DATA-005; TBD-031</x:v>
       </x:c>
     </x:row>
-    <x:row r="68" ht="32" customHeight="1">
+    <x:row r="68" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A68" s="22" t="str">
         <x:v>REQ-DATA-002</x:v>
       </x:c>
@@ -2396,7 +2399,7 @@
         <x:v>FS-CSV-002</x:v>
       </x:c>
       <x:c r="D68" s="9" t="str">
-        <x:v>ConfigurationLoader</x:v>
+        <x:v>DC-04 ConfigurationLoader</x:v>
       </x:c>
       <x:c r="E68" s="9" t="str">
         <x:v>인코딩·Quote·개행 오류 시험</x:v>
@@ -2409,7 +2412,7 @@
         <x:v>DATA-003,015~019</x:v>
       </x:c>
     </x:row>
-    <x:row r="69" ht="32" customHeight="1">
+    <x:row r="69" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A69" s="22" t="str">
         <x:v>REQ-DATA-003</x:v>
       </x:c>
@@ -2420,7 +2423,7 @@
         <x:v>FS-CSV-002</x:v>
       </x:c>
       <x:c r="D69" s="9" t="str">
-        <x:v>ConfigurationLoader</x:v>
+        <x:v>DC-04 ConfigurationLoader</x:v>
       </x:c>
       <x:c r="E69" s="9" t="str">
         <x:v>Header 별칭·순서·칼럼 수 오류 시험</x:v>
@@ -2433,7 +2436,7 @@
         <x:v>DATA-006,011; ERR-020,022</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" ht="32" customHeight="1">
+    <x:row r="70" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A70" s="22" t="str">
         <x:v>REQ-DATA-004</x:v>
       </x:c>
@@ -2444,7 +2447,7 @@
         <x:v>FS-CSV-002</x:v>
       </x:c>
       <x:c r="D70" s="9" t="str">
-        <x:v>ConfigurationLoader</x:v>
+        <x:v>DC-04 ConfigurationLoader</x:v>
       </x:c>
       <x:c r="E70" s="9" t="str">
         <x:v>숫자 문법·범위·NaN/Infinity 시험</x:v>
@@ -2457,7 +2460,7 @@
         <x:v>DATA-007~009; ERR-018,021</x:v>
       </x:c>
     </x:row>
-    <x:row r="71" ht="32" customHeight="1">
+    <x:row r="71" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A71" s="22" t="str">
         <x:v>REQ-DATA-005</x:v>
       </x:c>
@@ -2468,7 +2471,7 @@
         <x:v>FS-CSV-002</x:v>
       </x:c>
       <x:c r="D71" s="9" t="str">
-        <x:v>ConfigurationLoader</x:v>
+        <x:v>DC-04 ConfigurationLoader</x:v>
       </x:c>
       <x:c r="E71" s="9" t="str">
         <x:v>빈 Cell·공백·필수값 시험</x:v>
@@ -2481,7 +2484,7 @@
         <x:v>DATA-010~014</x:v>
       </x:c>
     </x:row>
-    <x:row r="72" ht="32" customHeight="1">
+    <x:row r="72" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A72" s="22" t="str">
         <x:v>REQ-DATA-006</x:v>
       </x:c>
@@ -2492,7 +2495,7 @@
         <x:v>FS-CSV-002,FS-DEV-001</x:v>
       </x:c>
       <x:c r="D72" s="9" t="str">
-        <x:v>ConfigurationLoader; DeviceRegistry</x:v>
+        <x:v>DC-04 ConfigurationLoader; DC-05 DeviceRegistry</x:v>
       </x:c>
       <x:c r="E72" s="9" t="str">
         <x:v>Schema와 Index/Port/Slave 유일성 시험</x:v>
@@ -2505,7 +2508,7 @@
         <x:v>DATA-DEV-001~006</x:v>
       </x:c>
     </x:row>
-    <x:row r="73" ht="32" customHeight="1">
+    <x:row r="73" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A73" s="22" t="str">
         <x:v>REQ-DATA-007</x:v>
       </x:c>
@@ -2516,7 +2519,7 @@
         <x:v>FS-CSV-002</x:v>
       </x:c>
       <x:c r="D73" s="9" t="str">
-        <x:v>ConfigurationLoader</x:v>
+        <x:v>DC-04 ConfigurationLoader</x:v>
       </x:c>
       <x:c r="E73" s="9" t="str">
         <x:v>Schema, Rule_ID, Quantity, 완전 중복 시험</x:v>
@@ -2529,7 +2532,7 @@
         <x:v>DATA-RULE-001~012</x:v>
       </x:c>
     </x:row>
-    <x:row r="74" ht="32" customHeight="1">
+    <x:row r="74" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A74" s="22" t="str">
         <x:v>REQ-DATA-008</x:v>
       </x:c>
@@ -2540,7 +2543,7 @@
         <x:v>FS-CSV-002</x:v>
       </x:c>
       <x:c r="D74" s="9" t="str">
-        <x:v>ConfigurationLoader</x:v>
+        <x:v>DC-04 ConfigurationLoader</x:v>
       </x:c>
       <x:c r="E74" s="9" t="str">
         <x:v>Rule 충돌 조합 시험</x:v>
@@ -2553,7 +2556,7 @@
         <x:v>DATA-RULE-007~010</x:v>
       </x:c>
     </x:row>
-    <x:row r="75" ht="32" customHeight="1">
+    <x:row r="75" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A75" s="22" t="str">
         <x:v>REQ-DATA-009</x:v>
       </x:c>
@@ -2564,7 +2567,7 @@
         <x:v>FS-CSV-002,FS-SIG-001</x:v>
       </x:c>
       <x:c r="D75" s="9" t="str">
-        <x:v>ConfigurationLoader; SignalCodec</x:v>
+        <x:v>DC-04 ConfigurationLoader; DC-07 SignalCodec</x:v>
       </x:c>
       <x:c r="E75" s="9" t="str">
         <x:v>Schema와 행 단위 검증 시험</x:v>
@@ -2577,7 +2580,7 @@
         <x:v>DATA-MAP-001~023</x:v>
       </x:c>
     </x:row>
-    <x:row r="76" ht="32" customHeight="1">
+    <x:row r="76" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A76" s="22" t="str">
         <x:v>REQ-DATA-010</x:v>
       </x:c>
@@ -2588,7 +2591,7 @@
         <x:v>FS-CSV-002,FS-SIG-001</x:v>
       </x:c>
       <x:c r="D76" s="9" t="str">
-        <x:v>ConfigurationLoader; SignalCodec</x:v>
+        <x:v>DC-04 ConfigurationLoader; DC-07 SignalCodec</x:v>
       </x:c>
       <x:c r="E76" s="9" t="str">
         <x:v>Enum 별칭·오타 거부 시험</x:v>
@@ -2601,7 +2604,7 @@
         <x:v>DATA-MAP-001~003</x:v>
       </x:c>
     </x:row>
-    <x:row r="77" ht="32" customHeight="1">
+    <x:row r="77" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A77" s="22" t="str">
         <x:v>REQ-DATA-011</x:v>
       </x:c>
@@ -2612,7 +2615,7 @@
         <x:v>FS-CSV-002</x:v>
       </x:c>
       <x:c r="D77" s="9" t="str">
-        <x:v>ConfigurationLoader</x:v>
+        <x:v>DC-04 ConfigurationLoader</x:v>
       </x:c>
       <x:c r="E77" s="9" t="str">
         <x:v>Value_Table 유무/내용 변경의 Runtime 불변 시험</x:v>
@@ -2625,7 +2628,7 @@
         <x:v>DATA-MAP-005,017~021</x:v>
       </x:c>
     </x:row>
-    <x:row r="78" ht="32" customHeight="1">
+    <x:row r="78" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A78" s="22" t="str">
         <x:v>REQ-DATA-012</x:v>
       </x:c>
@@ -2636,7 +2639,7 @@
         <x:v>FS-CSV-002</x:v>
       </x:c>
       <x:c r="D78" s="9" t="str">
-        <x:v>ConfigurationLoader</x:v>
+        <x:v>DC-04 ConfigurationLoader</x:v>
       </x:c>
       <x:c r="E78" s="9" t="str">
         <x:v>한도/초과 및 x86 Peak 메모리 시험</x:v>
@@ -2649,7 +2652,7 @@
         <x:v>IF-LIMIT-003; DATA-DEV-006; DATA-RULE-011; DATA-MAP-022</x:v>
       </x:c>
     </x:row>
-    <x:row r="79" ht="32" customHeight="1">
+    <x:row r="79" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A79" s="22" t="str">
         <x:v>REQ-DATA-013</x:v>
       </x:c>
@@ -2660,7 +2663,7 @@
         <x:v>FS-CSV-002</x:v>
       </x:c>
       <x:c r="D79" s="9" t="str">
-        <x:v>ConfigurationLoader</x:v>
+        <x:v>DC-04 ConfigurationLoader</x:v>
       </x:c>
       <x:c r="E79" s="9" t="str">
         <x:v>Byte 기반 한도·UTF-8 다중 Byte 시험</x:v>
@@ -2673,7 +2676,7 @@
         <x:v>IF-LIMIT-004~005; DATA-022~023</x:v>
       </x:c>
     </x:row>
-    <x:row r="80" ht="32" customHeight="1">
+    <x:row r="80" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A80" s="22" t="str">
         <x:v>REQ-DATA-014</x:v>
       </x:c>
@@ -2684,7 +2687,7 @@
         <x:v>FS-INIT-002</x:v>
       </x:c>
       <x:c r="D80" s="9" t="str">
-        <x:v>Build &amp; Packaging</x:v>
+        <x:v>DC-17 Build &amp; Packaging</x:v>
       </x:c>
       <x:c r="E80" s="9" t="str">
         <x:v>이동 가능한 Configuration 패키지 시험</x:v>
@@ -2697,7 +2700,7 @@
         <x:v>DATA-LAYOUT-001~004</x:v>
       </x:c>
     </x:row>
-    <x:row r="81" ht="32" customHeight="1">
+    <x:row r="81" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A81" s="22" t="str">
         <x:v>REQ-IF-001</x:v>
       </x:c>
@@ -2708,7 +2711,7 @@
         <x:v>FS-INIT-001</x:v>
       </x:c>
       <x:c r="D81" s="9" t="str">
-        <x:v>CAPL ABI Adapter</x:v>
+        <x:v>DC-01 CAPL ABI Adapter</x:v>
       </x:c>
       <x:c r="E81" s="9" t="str">
         <x:v>Vector Sample 기반 x86 최소 ABI 시험</x:v>
@@ -2721,7 +2724,7 @@
         <x:v>FACT-DLL-001~005; IF-ABI-009</x:v>
       </x:c>
     </x:row>
-    <x:row r="82" ht="32" customHeight="1">
+    <x:row r="82" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A82" s="22" t="str">
         <x:v>REQ-IF-002</x:v>
       </x:c>
@@ -2732,7 +2735,7 @@
         <x:v>FS-INIT-001</x:v>
       </x:c>
       <x:c r="D82" s="9" t="str">
-        <x:v>CAPL Core; CAPL ABI Adapter</x:v>
+        <x:v>DC-01 CAPL ABI Adapter; DC-13 CAPL Core</x:v>
       </x:c>
       <x:c r="E82" s="9" t="str">
         <x:v>Export Table 이름·Wrapper 호출 시험</x:v>
@@ -2745,7 +2748,7 @@
         <x:v>IF-NAME-001~003; IF-CTX-001~006</x:v>
       </x:c>
     </x:row>
-    <x:row r="83" ht="32" customHeight="1">
+    <x:row r="83" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A83" s="22" t="str">
         <x:v>REQ-IF-003</x:v>
       </x:c>
@@ -2756,7 +2759,7 @@
         <x:v>FS-INIT-001</x:v>
       </x:c>
       <x:c r="D83" s="9" t="str">
-        <x:v>CAPL ABI Adapter</x:v>
+        <x:v>DC-01 CAPL ABI Adapter</x:v>
       </x:c>
       <x:c r="E83" s="9" t="str">
         <x:v>최소 ABI Probe 및 Buffer 불변 시험</x:v>
@@ -2769,7 +2772,7 @@
         <x:v>IF-ABI-001~011</x:v>
       </x:c>
     </x:row>
-    <x:row r="84" ht="32" customHeight="1">
+    <x:row r="84" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A84" s="22" t="str">
         <x:v>REQ-IF-004</x:v>
       </x:c>
@@ -2780,7 +2783,7 @@
         <x:v>FS-INIT-001,FS-LIFE-001~004,FS-REG-001~003,FS-SIG-002~003,FS-MON-001~004,FS-DIAG-001~002</x:v>
       </x:c>
       <x:c r="D84" s="9" t="str">
-        <x:v>CAPL ABI Adapter</x:v>
+        <x:v>DC-01 CAPL ABI Adapter</x:v>
       </x:c>
       <x:c r="E84" s="9" t="str">
         <x:v>21개 Export Table/Wrapper Contract 시험</x:v>
@@ -2793,7 +2796,7 @@
         <x:v>IF-API-001~021</x:v>
       </x:c>
     </x:row>
-    <x:row r="85" ht="32" customHeight="1">
+    <x:row r="85" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A85" s="22" t="str">
         <x:v>REQ-IF-005</x:v>
       </x:c>
@@ -2804,7 +2807,7 @@
         <x:v>FS-LIFE-003,FS-DIAG-001</x:v>
       </x:c>
       <x:c r="D85" s="9" t="str">
-        <x:v>CAPL ABI Adapter; DiagnosticService</x:v>
+        <x:v>DC-01 CAPL ABI Adapter; DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E85" s="9" t="str">
         <x:v>동기/비동기/No Data 반환 시험</x:v>
@@ -2817,7 +2820,7 @@
         <x:v>IF-RET-001~009; IF-CODE-001~004</x:v>
       </x:c>
     </x:row>
-    <x:row r="86" ht="32" customHeight="1">
+    <x:row r="86" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A86" s="22" t="str">
         <x:v>REQ-IF-006</x:v>
       </x:c>
@@ -2828,7 +2831,7 @@
         <x:v>FS-REG-001~002,FS-SIG-002,FS-MON-003~004</x:v>
       </x:c>
       <x:c r="D86" s="9" t="str">
-        <x:v>CAPL Core; CAPL ABI Adapter</x:v>
+        <x:v>DC-01 CAPL ABI Adapter; DC-13 CAPL Core</x:v>
       </x:c>
       <x:c r="E86" s="9" t="str">
         <x:v>Buffer 부족·Embedded NUL·실패 시 출력 유지 시험</x:v>
@@ -2841,7 +2844,7 @@
         <x:v>IF-ABI-006~007,010~011; IF-RET-002~007</x:v>
       </x:c>
     </x:row>
-    <x:row r="87" ht="32" customHeight="1">
+    <x:row r="87" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A87" s="22" t="str">
         <x:v>REQ-IF-007</x:v>
       </x:c>
@@ -2852,7 +2855,7 @@
         <x:v>FS-MON-003~005</x:v>
       </x:c>
       <x:c r="D87" s="9" t="str">
-        <x:v>SnapshotService; CAPL Monitoring</x:v>
+        <x:v>DC-11 SnapshotService; DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E87" s="9" t="str">
         <x:v>Version·Capacity·필드 Routing 시험</x:v>
@@ -2865,7 +2868,7 @@
         <x:v>IF-META-001~016</x:v>
       </x:c>
     </x:row>
-    <x:row r="88" ht="32" customHeight="1">
+    <x:row r="88" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A88" s="22" t="str">
         <x:v>REQ-IF-008</x:v>
       </x:c>
@@ -2876,7 +2879,7 @@
         <x:v>FS-LIFE-003</x:v>
       </x:c>
       <x:c r="D88" s="9" t="str">
-        <x:v>LifecycleController</x:v>
+        <x:v>DC-03 LifecycleController</x:v>
       </x:c>
       <x:c r="E88" s="9" t="str">
         <x:v>상태 Snapshot 원자성과 Version 시험</x:v>
@@ -2889,7 +2892,7 @@
         <x:v>IF-LSTAT-001~014</x:v>
       </x:c>
     </x:row>
-    <x:row r="89" ht="32" customHeight="1">
+    <x:row r="89" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A89" s="22" t="str">
         <x:v>REQ-IF-009</x:v>
       </x:c>
@@ -2900,7 +2903,7 @@
         <x:v>FS-DIAG-001,FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D89" s="9" t="str">
-        <x:v>DiagnosticService; SnapshotService</x:v>
+        <x:v>DC-11 SnapshotService; DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E89" s="9" t="str">
         <x:v>Version·ValidMask·Capacity·NUL 시험</x:v>
@@ -2913,7 +2916,7 @@
         <x:v>IF-EMETA-001~025; IF-ESTAT-001~002; IF-CSTAT-001~002</x:v>
       </x:c>
     </x:row>
-    <x:row r="90" ht="32" customHeight="1">
+    <x:row r="90" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A90" s="22" t="str">
         <x:v>REQ-IF-010</x:v>
       </x:c>
@@ -2924,7 +2927,7 @@
         <x:v>FS-INIT-002,FS-COM-001,FS-DIAG-001</x:v>
       </x:c>
       <x:c r="D90" s="9" t="str">
-        <x:v>Generated Contracts</x:v>
+        <x:v>DC-16 Generated Contracts</x:v>
       </x:c>
       <x:c r="E90" s="9" t="str">
         <x:v>C++/CAPL 상수 목록 일치 시험</x:v>
@@ -2937,7 +2940,7 @@
         <x:v>IF-CONST-001~004; IF-ECLASS-001~004</x:v>
       </x:c>
     </x:row>
-    <x:row r="91" ht="32" customHeight="1">
+    <x:row r="91" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A91" s="22" t="str">
         <x:v>REQ-IF-011</x:v>
       </x:c>
@@ -2948,7 +2951,7 @@
         <x:v>FS-CSV-002,FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D91" s="9" t="str">
-        <x:v>Generated Contracts; ConfigurationLoader</x:v>
+        <x:v>DC-04 ConfigurationLoader; DC-16 Generated Contracts</x:v>
       </x:c>
       <x:c r="E91" s="9" t="str">
         <x:v>모든 한도 경계와 초과 시험</x:v>
@@ -2961,7 +2964,7 @@
         <x:v>IF-LIMIT-001~008</x:v>
       </x:c>
     </x:row>
-    <x:row r="92" ht="32" customHeight="1">
+    <x:row r="92" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A92" s="22" t="str">
         <x:v>REQ-IF-012</x:v>
       </x:c>
@@ -2972,7 +2975,7 @@
         <x:v>FS-REG-001,FS-REG-002</x:v>
       </x:c>
       <x:c r="D92" s="9" t="str">
-        <x:v>RegisterService; CAPL ABI Adapter</x:v>
+        <x:v>DC-01 CAPL ABI Adapter; DC-06 RegisterService</x:v>
       </x:c>
       <x:c r="E92" s="9" t="str">
         <x:v>Quantity/Capacity 조합 및 실패 불변 시험</x:v>
@@ -2985,7 +2988,7 @@
         <x:v>IF-REG-001~012</x:v>
       </x:c>
     </x:row>
-    <x:row r="93" ht="32" customHeight="1">
+    <x:row r="93" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A93" s="22" t="str">
         <x:v>REQ-IF-013</x:v>
       </x:c>
@@ -2996,7 +2999,7 @@
         <x:v>FS-SIG-002,FS-SIG-003</x:v>
       </x:c>
       <x:c r="D93" s="9" t="str">
-        <x:v>SignalCodec; CAPL ABI Adapter</x:v>
+        <x:v>DC-01 CAPL ABI Adapter; DC-07 SignalCodec</x:v>
       </x:c>
       <x:c r="E93" s="9" t="str">
         <x:v>정상/오류 시 Reference copy-restore 시험</x:v>
@@ -3009,7 +3012,7 @@
         <x:v>IF-SIG-001~007</x:v>
       </x:c>
     </x:row>
-    <x:row r="94" ht="32" customHeight="1">
+    <x:row r="94" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A94" s="22" t="str">
         <x:v>REQ-IF-014</x:v>
       </x:c>
@@ -3020,7 +3023,7 @@
         <x:v>FS-MON-003,FS-MON-004</x:v>
       </x:c>
       <x:c r="D94" s="9" t="str">
-        <x:v>SnapshotService; CAPL ABI Adapter</x:v>
+        <x:v>DC-01 CAPL ABI Adapter; DC-11 SnapshotService</x:v>
       </x:c>
       <x:c r="E94" s="9" t="str">
         <x:v>COM 비대기, Queue No Data, Buffer 부족 시험</x:v>
@@ -3033,7 +3036,7 @@
         <x:v>IF-MON-001~012</x:v>
       </x:c>
     </x:row>
-    <x:row r="95" ht="32" customHeight="1">
+    <x:row r="95" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A95" s="22" t="str">
         <x:v>REQ-ERR-001</x:v>
       </x:c>
@@ -3044,7 +3047,7 @@
         <x:v>FS-CSV-002,FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D95" s="9" t="str">
-        <x:v>ConfigurationLoader; DiagnosticService</x:v>
+        <x:v>DC-04 ConfigurationLoader; DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E95" s="9" t="str">
         <x:v>각 CSV 오류 강제 및 Context 정확성 시험</x:v>
@@ -3057,7 +3060,7 @@
         <x:v>ERR-009~023; LOG-009</x:v>
       </x:c>
     </x:row>
-    <x:row r="96" ht="32" customHeight="1">
+    <x:row r="96" ht="43.20000076293945" hidden="0" customHeight="1">
       <x:c r="A96" s="22" t="str">
         <x:v>REQ-ERR-002</x:v>
       </x:c>
@@ -3068,7 +3071,7 @@
         <x:v>FS-CSV-003,FS-REG-001~003,FS-SIG-002~004</x:v>
       </x:c>
       <x:c r="D96" s="9" t="str">
-        <x:v>All core services</x:v>
+        <x:v>DC-01 CAPL ABI Adapter; DC-04 ConfigurationLoader; DC-06 RegisterService; DC-07 SignalCodec; DC-11 SnapshotService; DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E96" s="9" t="str">
         <x:v>실패 주입 및 전후 메모리 비교 시험</x:v>
@@ -3081,7 +3084,7 @@
         <x:v>ERR-001~007,010~018,024~036,042</x:v>
       </x:c>
     </x:row>
-    <x:row r="97" ht="32" customHeight="1">
+    <x:row r="97" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A97" s="22" t="str">
         <x:v>REQ-ERR-003</x:v>
       </x:c>
@@ -3092,7 +3095,7 @@
         <x:v>FS-MODBUS-005</x:v>
       </x:c>
       <x:c r="D97" s="9" t="str">
-        <x:v>ModbusRtuEngine</x:v>
+        <x:v>DC-08 ModbusRtuEngine</x:v>
       </x:c>
       <x:c r="E97" s="9" t="str">
         <x:v>Exception Golden Vector 시험</x:v>
@@ -3105,7 +3108,7 @@
         <x:v>ERR-039~043; FR-RTU-033</x:v>
       </x:c>
     </x:row>
-    <x:row r="98" ht="32" customHeight="1">
+    <x:row r="98" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A98" s="22" t="str">
         <x:v>REQ-ERR-004</x:v>
       </x:c>
@@ -3116,7 +3119,7 @@
         <x:v>FS-DIAG-001,FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D98" s="9" t="str">
-        <x:v>DiagnosticService</x:v>
+        <x:v>DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E98" s="9" t="str">
         <x:v>영역별 오류와 OsError 분리 시험</x:v>
@@ -3129,7 +3132,7 @@
         <x:v>IF-CODE-005~016</x:v>
       </x:c>
     </x:row>
-    <x:row r="99" ht="32" customHeight="1">
+    <x:row r="99" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A99" s="22" t="str">
         <x:v>REQ-ERR-005</x:v>
       </x:c>
@@ -3140,7 +3143,7 @@
         <x:v>FS-DIAG-001,FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D99" s="9" t="str">
-        <x:v>Generated Contracts</x:v>
+        <x:v>DC-16 Generated Contracts</x:v>
       </x:c>
       <x:c r="E99" s="9" t="str">
         <x:v>90개 목록 일치 및 신규 코드 추가 회귀 시험</x:v>
@@ -3153,7 +3156,7 @@
         <x:v>IF-CODE-017~020; TBD-064</x:v>
       </x:c>
     </x:row>
-    <x:row r="100" ht="32" customHeight="1">
+    <x:row r="100" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A100" s="22" t="str">
         <x:v>REQ-ERR-006</x:v>
       </x:c>
@@ -3164,7 +3167,7 @@
         <x:v>FS-DIAG-001,FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D100" s="9" t="str">
-        <x:v>DiagnosticService</x:v>
+        <x:v>DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E100" s="9" t="str">
         <x:v>동시 오류·Context 격리·Polling 시험</x:v>
@@ -3177,7 +3180,7 @@
         <x:v>IF-ERR-001~015; DES-ERR-001~004</x:v>
       </x:c>
     </x:row>
-    <x:row r="101" ht="32" customHeight="1">
+    <x:row r="101" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A101" s="22" t="str">
         <x:v>REQ-ERR-007</x:v>
       </x:c>
@@ -3188,7 +3191,7 @@
         <x:v>FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D101" s="9" t="str">
-        <x:v>DiagnosticService</x:v>
+        <x:v>DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E101" s="9" t="str">
         <x:v>반복 Noise·Overflow·Sequence 시험</x:v>
@@ -3201,7 +3204,7 @@
         <x:v>ERR-032~033,040; LOG-011~013</x:v>
       </x:c>
     </x:row>
-    <x:row r="102" ht="32" customHeight="1">
+    <x:row r="102" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A102" s="22" t="str">
         <x:v>REQ-ERR-008</x:v>
       </x:c>
@@ -3212,7 +3215,7 @@
         <x:v>FS-LIFE-001,FS-LIFE-004</x:v>
       </x:c>
       <x:c r="D102" s="9" t="str">
-        <x:v>LifecycleController</x:v>
+        <x:v>DC-03 LifecycleController</x:v>
       </x:c>
       <x:c r="E102" s="9" t="str">
         <x:v>실패 등급별 상태 전이 시험</x:v>
@@ -3225,7 +3228,7 @@
         <x:v>FR-LIFE-013; ERR-028,034~038</x:v>
       </x:c>
     </x:row>
-    <x:row r="103" ht="32" customHeight="1">
+    <x:row r="103" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A103" s="22" t="str">
         <x:v>REQ-PERF-001</x:v>
       </x:c>
@@ -3236,7 +3239,7 @@
         <x:v>FS-MODBUS-002~004</x:v>
       </x:c>
       <x:c r="D103" s="9" t="str">
-        <x:v>PortWorker; ModbusRtuEngine</x:v>
+        <x:v>DC-08 ModbusRtuEngine; DC-10 PortWorker</x:v>
       </x:c>
       <x:c r="E103" s="9" t="str">
         <x:v>회사 환경 실제 Timeout 기반 지연 측정</x:v>
@@ -3249,7 +3252,7 @@
         <x:v>PERF-001~003; TBD-039</x:v>
       </x:c>
     </x:row>
-    <x:row r="104" ht="32" customHeight="1">
+    <x:row r="104" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A104" s="22" t="str">
         <x:v>REQ-PERF-002</x:v>
       </x:c>
@@ -3260,7 +3263,7 @@
         <x:v>FS-MON-003,FS-MON-004,FS-MON-006</x:v>
       </x:c>
       <x:c r="D104" s="9" t="str">
-        <x:v>CAPL Monitoring</x:v>
+        <x:v>DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E104" s="9" t="str">
         <x:v>Trace Timestamp 기반 지연 측정</x:v>
@@ -3273,7 +3276,7 @@
         <x:v>PERF-004~013; TBD-039</x:v>
       </x:c>
     </x:row>
-    <x:row r="105" ht="32" customHeight="1">
+    <x:row r="105" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A105" s="22" t="str">
         <x:v>REQ-PERF-003</x:v>
       </x:c>
@@ -3284,7 +3287,7 @@
         <x:v>FS-INIT-001,FS-LIFE-001~003,FS-MON-003~004</x:v>
       </x:c>
       <x:c r="D105" s="9" t="str">
-        <x:v>CAPL ABI Adapter</x:v>
+        <x:v>DC-01 CAPL ABI Adapter</x:v>
       </x:c>
       <x:c r="E105" s="9" t="str">
         <x:v>호출시간 계측과 정적 코드 검토</x:v>
@@ -3297,7 +3300,7 @@
         <x:v>NFR-007,010</x:v>
       </x:c>
     </x:row>
-    <x:row r="106" ht="32" customHeight="1">
+    <x:row r="106" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A106" s="22" t="str">
         <x:v>REQ-PERF-004</x:v>
       </x:c>
@@ -3308,7 +3311,7 @@
         <x:v>FS-MON-002,FS-MON-006</x:v>
       </x:c>
       <x:c r="D106" s="9" t="str">
-        <x:v>CAPL Monitoring</x:v>
+        <x:v>DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E106" s="9" t="str">
         <x:v>200 Rule 최대/대표 부하 시험</x:v>
@@ -3321,7 +3324,7 @@
         <x:v>FR-LOAD-012~014,019; PERF-014~019</x:v>
       </x:c>
     </x:row>
-    <x:row r="107" ht="32" customHeight="1">
+    <x:row r="107" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A107" s="22" t="str">
         <x:v>REQ-PERF-005</x:v>
       </x:c>
@@ -3332,7 +3335,7 @@
         <x:v>FS-CSV-003</x:v>
       </x:c>
       <x:c r="D107" s="9" t="str">
-        <x:v>DeviceRegistry; ConfigurationLoader</x:v>
+        <x:v>DC-04 ConfigurationLoader; DC-05 DeviceRegistry</x:v>
       </x:c>
       <x:c r="E107" s="9" t="str">
         <x:v>Peak Working Set 측정</x:v>
@@ -3345,7 +3348,7 @@
         <x:v>PERF-018</x:v>
       </x:c>
     </x:row>
-    <x:row r="108" ht="32" customHeight="1">
+    <x:row r="108" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A108" s="22" t="str">
         <x:v>REQ-PERF-006</x:v>
       </x:c>
@@ -3356,7 +3359,7 @@
         <x:v>FS-SHUT-001</x:v>
       </x:c>
       <x:c r="D108" s="9" t="str">
-        <x:v>LifecycleController</x:v>
+        <x:v>DC-03 LifecycleController</x:v>
       </x:c>
       <x:c r="E108" s="9" t="str">
         <x:v>각 상태 Finalize 시간 및 지연 Driver 시험</x:v>
@@ -3369,7 +3372,7 @@
         <x:v>PERF-020~022; TBD-065</x:v>
       </x:c>
     </x:row>
-    <x:row r="109" ht="32" customHeight="1">
+    <x:row r="109" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A109" s="22" t="str">
         <x:v>REQ-REL-001</x:v>
       </x:c>
@@ -3380,7 +3383,7 @@
         <x:v>FS-COM-002,FS-MODBUS-001</x:v>
       </x:c>
       <x:c r="D109" s="9" t="str">
-        <x:v>PortWorker</x:v>
+        <x:v>DC-10 PortWorker</x:v>
       </x:c>
       <x:c r="E109" s="9" t="str">
         <x:v>동시 두 Port I/O와 Handle 소유 검토</x:v>
@@ -3393,7 +3396,7 @@
         <x:v>DES-THREAD-001</x:v>
       </x:c>
     </x:row>
-    <x:row r="110" ht="32" customHeight="1">
+    <x:row r="110" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A110" s="22" t="str">
         <x:v>REQ-REL-002</x:v>
       </x:c>
@@ -3404,7 +3407,7 @@
         <x:v>FS-REG-001~003,FS-MON-004,FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D110" s="9" t="str">
-        <x:v>RegisterService; SnapshotService; DiagnosticService</x:v>
+        <x:v>DC-06 RegisterService; DC-11 SnapshotService; DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E110" s="9" t="str">
         <x:v>동시 RTU/CAPL 접근 및 Race 시험</x:v>
@@ -3417,7 +3420,7 @@
         <x:v>DES-THREAD-002~003</x:v>
       </x:c>
     </x:row>
-    <x:row r="111" ht="32" customHeight="1">
+    <x:row r="111" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A111" s="22" t="str">
         <x:v>REQ-REL-003</x:v>
       </x:c>
@@ -3428,7 +3431,7 @@
         <x:v>FS-REG-002,FS-SHUT-001</x:v>
       </x:c>
       <x:c r="D111" s="9" t="str">
-        <x:v>All runtime services</x:v>
+        <x:v>DC-03 LifecycleController; DC-06 RegisterService; DC-11 SnapshotService; DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E111" s="9" t="str">
         <x:v>Deadlock Stress 및 Lock-order 검토</x:v>
@@ -3441,7 +3444,7 @@
         <x:v>DES-THREAD-004</x:v>
       </x:c>
     </x:row>
-    <x:row r="112" ht="32" customHeight="1">
+    <x:row r="112" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A112" s="22" t="str">
         <x:v>REQ-REL-004</x:v>
       </x:c>
@@ -3452,7 +3455,7 @@
         <x:v>FS-MON-004,FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D112" s="9" t="str">
-        <x:v>SnapshotService; DiagnosticService</x:v>
+        <x:v>DC-11 SnapshotService; DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E112" s="9" t="str">
         <x:v>Allocator hook/Stress 시험</x:v>
@@ -3465,7 +3468,7 @@
         <x:v>DES-THREAD-003; DES-CAN-011~012</x:v>
       </x:c>
     </x:row>
-    <x:row r="113" ht="32" customHeight="1">
+    <x:row r="113" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A113" s="22" t="str">
         <x:v>REQ-REL-005</x:v>
       </x:c>
@@ -3476,7 +3479,7 @@
         <x:v>FS-MON-003,FS-MON-004</x:v>
       </x:c>
       <x:c r="D113" s="9" t="str">
-        <x:v>RegisterService; SnapshotService</x:v>
+        <x:v>DC-06 RegisterService; DC-11 SnapshotService</x:v>
       </x:c>
       <x:c r="E113" s="9" t="str">
         <x:v>동시 다중 Register Write와 Snapshot 일관성 시험</x:v>
@@ -3489,7 +3492,7 @@
         <x:v>IF-MON-002~003</x:v>
       </x:c>
     </x:row>
-    <x:row r="114" ht="32" customHeight="1">
+    <x:row r="114" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A114" s="22" t="str">
         <x:v>REQ-REL-006</x:v>
       </x:c>
@@ -3500,7 +3503,7 @@
         <x:v>FS-MON-004,FS-MON-006</x:v>
       </x:c>
       <x:c r="D114" s="9" t="str">
-        <x:v>SnapshotService; CAPL Monitoring</x:v>
+        <x:v>DC-11 SnapshotService; DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E114" s="9" t="str">
         <x:v>Burst/Overflow 중 RTU 응답 시험</x:v>
@@ -3513,7 +3516,7 @@
         <x:v>NFR-002~004; FR-LOAD-009</x:v>
       </x:c>
     </x:row>
-    <x:row r="115" ht="32" customHeight="1">
+    <x:row r="115" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A115" s="22" t="str">
         <x:v>REQ-RES-001</x:v>
       </x:c>
@@ -3524,7 +3527,7 @@
         <x:v>FS-DEV-001</x:v>
       </x:c>
       <x:c r="D115" s="9" t="str">
-        <x:v>DeviceRegistry</x:v>
+        <x:v>DC-05 DeviceRegistry</x:v>
       </x:c>
       <x:c r="E115" s="9" t="str">
         <x:v>Device 수별 메모리 및 직접 Address 시험</x:v>
@@ -3537,7 +3540,7 @@
         <x:v>DES-REG-005</x:v>
       </x:c>
     </x:row>
-    <x:row r="116" ht="32" customHeight="1">
+    <x:row r="116" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A116" s="22" t="str">
         <x:v>REQ-RES-002</x:v>
       </x:c>
@@ -3548,7 +3551,7 @@
         <x:v>FS-SHUT-001</x:v>
       </x:c>
       <x:c r="D116" s="9" t="str">
-        <x:v>LifecycleController</x:v>
+        <x:v>DC-03 LifecycleController</x:v>
       </x:c>
       <x:c r="E116" s="9" t="str">
         <x:v>Thread/Handle 누수와 종료 Race 시험</x:v>
@@ -3561,7 +3564,7 @@
         <x:v>FR-LIFE-018~019; DES-THREAD-005</x:v>
       </x:c>
     </x:row>
-    <x:row r="117" ht="32" customHeight="1">
+    <x:row r="117" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A117" s="22" t="str">
         <x:v>REQ-RES-003</x:v>
       </x:c>
@@ -3572,7 +3575,7 @@
         <x:v>FS-MON-003,FS-MON-004,FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D117" s="9" t="str">
-        <x:v>SnapshotService; DiagnosticService</x:v>
+        <x:v>DC-11 SnapshotService; DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E117" s="9" t="str">
         <x:v>Capacity 경계와 Overflow 정책 시험</x:v>
@@ -3585,7 +3588,7 @@
         <x:v>IF-LIMIT-006</x:v>
       </x:c>
     </x:row>
-    <x:row r="118" ht="32" customHeight="1">
+    <x:row r="118" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A118" s="22" t="str">
         <x:v>REQ-RES-004</x:v>
       </x:c>
@@ -3596,7 +3599,7 @@
         <x:v>FS-MON-004,FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D118" s="9" t="str">
-        <x:v>SnapshotService; DiagnosticService</x:v>
+        <x:v>DC-11 SnapshotService; DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E118" s="9" t="str">
         <x:v>포화 및 Sequence wrap 시험</x:v>
@@ -3609,7 +3612,7 @@
         <x:v>IF-QSTAT-001~004</x:v>
       </x:c>
     </x:row>
-    <x:row r="119" ht="32" customHeight="1">
+    <x:row r="119" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A119" s="22" t="str">
         <x:v>REQ-DIAG-001</x:v>
       </x:c>
@@ -3620,7 +3623,7 @@
         <x:v>FS-DIAG-001</x:v>
       </x:c>
       <x:c r="D119" s="9" t="str">
-        <x:v>CAPL Core; DiagnosticService</x:v>
+        <x:v>DC-12 DiagnosticService; DC-13 CAPL Core</x:v>
       </x:c>
       <x:c r="E119" s="9" t="str">
         <x:v>오류별 Write Window 출력 시험</x:v>
@@ -3633,7 +3636,7 @@
         <x:v>LOG-004,009~010</x:v>
       </x:c>
     </x:row>
-    <x:row r="120" ht="32" customHeight="1">
+    <x:row r="120" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A120" s="22" t="str">
         <x:v>REQ-DIAG-002</x:v>
       </x:c>
@@ -3644,7 +3647,7 @@
         <x:v>FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D120" s="9" t="str">
-        <x:v>CAPL Core; DiagnosticService</x:v>
+        <x:v>DC-12 DiagnosticService; DC-13 CAPL Core</x:v>
       </x:c>
       <x:c r="E120" s="9" t="str">
         <x:v>비동기 오류 순서·병합·Overflow 출력 시험</x:v>
@@ -3657,7 +3660,7 @@
         <x:v>LOG-011~013</x:v>
       </x:c>
     </x:row>
-    <x:row r="121" ht="32" customHeight="1">
+    <x:row r="121" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A121" s="22" t="str">
         <x:v>REQ-DIAG-003</x:v>
       </x:c>
@@ -3668,7 +3671,7 @@
         <x:v>FS-MON-006,FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D121" s="9" t="str">
-        <x:v>CAPL Monitoring; DiagnosticService</x:v>
+        <x:v>DC-12 DiagnosticService; DC-14 CAPL Monitoring</x:v>
       </x:c>
       <x:c r="E121" s="9" t="str">
         <x:v>부하 시험 진단값 상호 검증</x:v>
@@ -3681,7 +3684,7 @@
         <x:v>LOG-002~008,014~017</x:v>
       </x:c>
     </x:row>
-    <x:row r="122" ht="32" customHeight="1">
+    <x:row r="122" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A122" s="22" t="str">
         <x:v>REQ-DIAG-004</x:v>
       </x:c>
@@ -3692,7 +3695,7 @@
         <x:v>FS-LIFE-001,FS-LIFE-004,FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D122" s="9" t="str">
-        <x:v>Win32SerialPort; DiagnosticService</x:v>
+        <x:v>DC-09 Win32SerialPort; DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E122" s="9" t="str">
         <x:v>강제 Win32 오류와 Context 시험</x:v>
@@ -3705,7 +3708,7 @@
         <x:v>ERR-027~038; LOG-013</x:v>
       </x:c>
     </x:row>
-    <x:row r="123" ht="32" customHeight="1">
+    <x:row r="123" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A123" s="22" t="str">
         <x:v>REQ-DIAG-005</x:v>
       </x:c>
@@ -3716,7 +3719,7 @@
         <x:v>FS-COM-003,FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D123" s="9" t="str">
-        <x:v>DiagnosticService</x:v>
+        <x:v>DC-12 DiagnosticService</x:v>
       </x:c>
       <x:c r="E123" s="9" t="str">
         <x:v>반복 동일 오류 부하 시험</x:v>
@@ -3729,7 +3732,7 @@
         <x:v>ERR-040; LOG-011</x:v>
       </x:c>
     </x:row>
-    <x:row r="124" ht="32" customHeight="1">
+    <x:row r="124" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A124" s="22" t="str">
         <x:v>REQ-COMP-001</x:v>
       </x:c>
@@ -3740,7 +3743,7 @@
         <x:v>FS-INIT-001</x:v>
       </x:c>
       <x:c r="D124" s="9" t="str">
-        <x:v>Build &amp; Packaging</x:v>
+        <x:v>DC-17 Build &amp; Packaging</x:v>
       </x:c>
       <x:c r="E124" s="9" t="str">
         <x:v>깨끗한 PC Win32 Build 및 CANalyzer 로딩 시험</x:v>
@@ -3753,7 +3756,7 @@
         <x:v>ENV-001~002,010~011; COMP-001~002,008</x:v>
       </x:c>
     </x:row>
-    <x:row r="125" ht="32" customHeight="1">
+    <x:row r="125" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A125" s="22" t="str">
         <x:v>REQ-COMP-002</x:v>
       </x:c>
@@ -3764,7 +3767,7 @@
         <x:v>FS-INIT-001</x:v>
       </x:c>
       <x:c r="D125" s="9" t="str">
-        <x:v>Build &amp; Packaging</x:v>
+        <x:v>DC-17 Build &amp; Packaging</x:v>
       </x:c>
       <x:c r="E125" s="9" t="str">
         <x:v>설치 경로 변경·Clean Build 시험</x:v>
@@ -3777,7 +3780,7 @@
         <x:v>DES-BUILD-001~005; TBD-059</x:v>
       </x:c>
     </x:row>
-    <x:row r="126" ht="32" customHeight="1">
+    <x:row r="126" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A126" s="22" t="str">
         <x:v>REQ-COMP-003</x:v>
       </x:c>
@@ -3788,7 +3791,7 @@
         <x:v>FS-INIT-001</x:v>
       </x:c>
       <x:c r="D126" s="9" t="str">
-        <x:v>Build &amp; Packaging</x:v>
+        <x:v>DC-17 Build &amp; Packaging</x:v>
       </x:c>
       <x:c r="E126" s="9" t="str">
         <x:v>공개 Export/문서에 Legacy 이름 부재 검토</x:v>
@@ -3801,7 +3804,7 @@
         <x:v>PRJ-005~006; COMP-009~010</x:v>
       </x:c>
     </x:row>
-    <x:row r="127" ht="32" customHeight="1">
+    <x:row r="127" ht="54" hidden="0" customHeight="1">
       <x:c r="A127" s="22" t="str">
         <x:v>REQ-COMP-004</x:v>
       </x:c>
@@ -3812,7 +3815,7 @@
         <x:v>FS-INIT-001</x:v>
       </x:c>
       <x:c r="D127" s="9" t="str">
-        <x:v>M485E.Core</x:v>
+        <x:v>DC-04 ConfigurationLoader; DC-05 DeviceRegistry; DC-06 RegisterService; DC-07 SignalCodec; DC-08 ModbusRtuEngine; DC-11 SnapshotService; DC-12 DiagnosticService; DC-17 Build &amp; Packaging</x:v>
       </x:c>
       <x:c r="E127" s="9" t="str">
         <x:v>Win32 타입 크기 검토; x64는 후속 체크리스트</x:v>
@@ -3825,7 +3828,7 @@
         <x:v>ENV-011; FUT-001~005</x:v>
       </x:c>
     </x:row>
-    <x:row r="128" ht="32" customHeight="1">
+    <x:row r="128" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A128" s="22" t="str">
         <x:v>REQ-COMP-005</x:v>
       </x:c>
@@ -3836,7 +3839,7 @@
         <x:v>FS-COM-002,FS-COM-003,FS-MODBUS-002~005</x:v>
       </x:c>
       <x:c r="D128" s="9" t="str">
-        <x:v>ModbusRtuEngine</x:v>
+        <x:v>DC-08 ModbusRtuEngine</x:v>
       </x:c>
       <x:c r="E128" s="9" t="str">
         <x:v>공식 Protocol Vector 및 경계 시험</x:v>
@@ -3849,7 +3852,7 @@
         <x:v>COMP-013</x:v>
       </x:c>
     </x:row>
-    <x:row r="129" ht="32" customHeight="1">
+    <x:row r="129" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A129" s="22" t="str">
         <x:v>REQ-COMP-006</x:v>
       </x:c>
@@ -3860,7 +3863,7 @@
         <x:v>FS-DIAG-001,FS-DIAG-002</x:v>
       </x:c>
       <x:c r="D129" s="9" t="str">
-        <x:v>Generated Contracts</x:v>
+        <x:v>DC-16 Generated Contracts</x:v>
       </x:c>
       <x:c r="E129" s="9" t="str">
         <x:v>구 Layout consumer 회귀 시험</x:v>
@@ -3873,7 +3876,7 @@
         <x:v>IF-META-015; IF-QSTAT-004; IF-LIMIT-008; IF-CODE-017</x:v>
       </x:c>
     </x:row>
-    <x:row r="130" ht="32" customHeight="1">
+    <x:row r="130" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A130" s="22" t="str">
         <x:v>REQ-SEC-001</x:v>
       </x:c>
@@ -3884,7 +3887,7 @@
         <x:v>FS-CSV-001,FS-CSV-002</x:v>
       </x:c>
       <x:c r="D130" s="9" t="str">
-        <x:v>ConfigurationLoader</x:v>
+        <x:v>DC-04 ConfigurationLoader</x:v>
       </x:c>
       <x:c r="E130" s="9" t="str">
         <x:v>로컬/UNC/권한 부족 경로 시험</x:v>
@@ -3897,7 +3900,7 @@
         <x:v>NFR-012; COMP-006; OOS-015</x:v>
       </x:c>
     </x:row>
-    <x:row r="131" ht="32" customHeight="1">
+    <x:row r="131" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A131" s="22" t="str">
         <x:v>REQ-SEC-002</x:v>
       </x:c>
@@ -3908,7 +3911,7 @@
         <x:v>FS-MODBUS-001</x:v>
       </x:c>
       <x:c r="D131" s="9" t="str">
-        <x:v>System boundary</x:v>
+        <x:v>DC-08 ModbusRtuEngine; DC-10 PortWorker</x:v>
       </x:c>
       <x:c r="E131" s="9" t="str">
         <x:v>보안 경계 문서 검토</x:v>
@@ -3921,7 +3924,7 @@
         <x:v>NFR-012</x:v>
       </x:c>
     </x:row>
-    <x:row r="132" ht="32" customHeight="1">
+    <x:row r="132" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A132" s="22" t="str">
         <x:v>REQ-SEC-003</x:v>
       </x:c>
@@ -3932,7 +3935,7 @@
         <x:v>FS-CSV-001,FS-DIAG-001</x:v>
       </x:c>
       <x:c r="D132" s="9" t="str">
-        <x:v>CAPL ABI Adapter; ConfigurationLoader</x:v>
+        <x:v>DC-01 CAPL ABI Adapter; DC-04 ConfigurationLoader</x:v>
       </x:c>
       <x:c r="E132" s="9" t="str">
         <x:v>ASCII/한글 경로·Text round-trip 시험</x:v>
@@ -3953,7 +3956,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6578c94867b04602"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R225405ba02354d1c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7010,7 +7013,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd170a116ed7b4dae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R100a34472a584bbc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7024,7 +7027,7 @@
     <x:col min="3" max="3" width="80" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A1" s="21" t="str">
         <x:v>Functional Specification ID</x:v>
       </x:c>
@@ -7035,7 +7038,7 @@
         <x:v>Covered Requirement IDs</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="32" customHeight="1">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="9" t="str">
         <x:v>FS-INIT-001</x:v>
       </x:c>
@@ -7043,10 +7046,10 @@
         <x:v>CAPL DLL 초기화</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>REQ-FUNC-001; REQ-IF-001~003; REQ-COMP-001~004</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-001; REQ-IF-001~004; REQ-PERF-003; REQ-COMP-001~004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="9" t="str">
         <x:v>FS-INIT-002</x:v>
       </x:c>
@@ -7054,10 +7057,10 @@
         <x:v>Configuration 입력 준비</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>REQ-FUNC-009~010; REQ-DATA-014; REQ-IF-010</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="32" customHeight="1">
+        <x:v>REQ-DATA-014; REQ-IF-010</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="9" t="str">
         <x:v>FS-CSV-001</x:v>
       </x:c>
@@ -7065,10 +7068,10 @@
         <x:v>CSV 경로 처리</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>REQ-FUNC-009~010; REQ-SEC-001,REQ-SEC-003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-009~010; REQ-SEC-001, REQ-SEC-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="9" t="str">
         <x:v>FS-CSV-002</x:v>
       </x:c>
@@ -7076,10 +7079,10 @@
         <x:v>CSV Parsing 및 전체 검증</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>REQ-FUNC-011; REQ-DATA-001~013; REQ-ERR-001~002</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-011, REQ-FUNC-026; REQ-DATA-001~013; REQ-IF-011; REQ-ERR-001; REQ-SEC-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="9" t="str">
         <x:v>FS-CSV-003</x:v>
       </x:c>
@@ -7087,10 +7090,10 @@
         <x:v>원자적 Refresh</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
-        <x:v>REQ-FUNC-011~013; REQ-PERF-005</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-011~013; REQ-ERR-002; REQ-PERF-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="9" t="str">
         <x:v>FS-LIFE-001</x:v>
       </x:c>
@@ -7098,10 +7101,10 @@
         <x:v>전체 Connect</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
-        <x:v>REQ-FUNC-002~004; REQ-COM-002~004</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-002, REQ-FUNC-004; REQ-IF-004; REQ-ERR-008; REQ-PERF-003; REQ-DIAG-004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="9" t="str">
         <x:v>FS-LIFE-002</x:v>
       </x:c>
@@ -7109,10 +7112,10 @@
         <x:v>전체 Disconnect</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>REQ-FUNC-002,REQ-FUNC-005</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-002, REQ-FUNC-005; REQ-IF-004; REQ-PERF-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="9" t="str">
         <x:v>FS-LIFE-003</x:v>
       </x:c>
@@ -7120,10 +7123,10 @@
         <x:v>Lifecycle 상태 Polling</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
-        <x:v>REQ-FUNC-002~003; REQ-IF-005,REQ-IF-008</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-002~003; REQ-IF-004~005, REQ-IF-008; REQ-PERF-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="9" t="str">
         <x:v>FS-LIFE-004</x:v>
       </x:c>
@@ -7131,10 +7134,10 @@
         <x:v>치명적 COM 장애 복구</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>REQ-FUNC-006~007; REQ-ERR-008</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-006~007; REQ-IF-004; REQ-ERR-008; REQ-DIAG-004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="9" t="str">
         <x:v>FS-COM-001</x:v>
       </x:c>
@@ -7142,10 +7145,10 @@
         <x:v>Serial Port 설정</x:v>
       </x:c>
       <x:c r="C11" s="9" t="str">
-        <x:v>REQ-COM-001~005</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="32" customHeight="1">
+        <x:v>REQ-COM-001~005; REQ-IF-010</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="9" t="str">
         <x:v>FS-COM-002</x:v>
       </x:c>
@@ -7153,10 +7156,10 @@
         <x:v>RTU Stream Frame 조립</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
-        <x:v>REQ-COM-012~013; REQ-REL-001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="32" customHeight="1">
+        <x:v>REQ-COM-012~013; REQ-REL-001; REQ-COMP-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="9" t="str">
         <x:v>FS-COM-003</x:v>
       </x:c>
@@ -7164,10 +7167,10 @@
         <x:v>RTU Frame 및 CRC 검증</x:v>
       </x:c>
       <x:c r="C13" s="9" t="str">
-        <x:v>REQ-COM-011,REQ-COM-014; REQ-DIAG-005</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="32" customHeight="1">
+        <x:v>REQ-COM-011, REQ-COM-014; REQ-DIAG-005; REQ-COMP-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="9" t="str">
         <x:v>FS-MODBUS-001</x:v>
       </x:c>
@@ -7175,10 +7178,10 @@
         <x:v>Slave Routing</x:v>
       </x:c>
       <x:c r="C14" s="9" t="str">
-        <x:v>REQ-FUNC-014; REQ-COM-010,REQ-COM-015; REQ-SEC-002</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="32" customHeight="1">
+        <x:v>REQ-COM-010, REQ-COM-015; REQ-REL-001; REQ-SEC-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="9" t="str">
         <x:v>FS-MODBUS-002</x:v>
       </x:c>
@@ -7186,10 +7189,10 @@
         <x:v>FC03 처리</x:v>
       </x:c>
       <x:c r="C15" s="9" t="str">
-        <x:v>REQ-COM-006~008,REQ-COM-011; REQ-DATA-001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="32" customHeight="1">
+        <x:v>REQ-COM-006~008; REQ-DATA-001; REQ-PERF-001; REQ-COMP-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="9" t="str">
         <x:v>FS-MODBUS-003</x:v>
       </x:c>
@@ -7197,10 +7200,10 @@
         <x:v>FC04 처리</x:v>
       </x:c>
       <x:c r="C16" s="9" t="str">
-        <x:v>REQ-COM-006~008,REQ-COM-011; REQ-DATA-001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="32" customHeight="1">
+        <x:v>REQ-COM-006~008; REQ-DATA-001; REQ-PERF-001; REQ-COMP-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="9" t="str">
         <x:v>FS-MODBUS-004</x:v>
       </x:c>
@@ -7208,10 +7211,10 @@
         <x:v>FC10 처리</x:v>
       </x:c>
       <x:c r="C17" s="9" t="str">
-        <x:v>REQ-COM-006~009; REQ-FUNC-018</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="32" customHeight="1">
+        <x:v>REQ-COM-006~009; REQ-DATA-001; REQ-PERF-001; REQ-COMP-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="9" t="str">
         <x:v>FS-MODBUS-005</x:v>
       </x:c>
@@ -7219,10 +7222,10 @@
         <x:v>무응답 및 Exception 처리</x:v>
       </x:c>
       <x:c r="C18" s="9" t="str">
-        <x:v>REQ-COM-006~010,REQ-COM-014; REQ-ERR-003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="32" customHeight="1">
+        <x:v>REQ-COM-006~007, REQ-COM-010, REQ-COM-014; REQ-ERR-003; REQ-COMP-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="9" t="str">
         <x:v>FS-DEV-001</x:v>
       </x:c>
@@ -7230,10 +7233,10 @@
         <x:v>Device Registry 구성</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
-        <x:v>REQ-FUNC-014; REQ-DATA-006,REQ-DATA-012; REQ-RES-001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-014; REQ-DATA-006; REQ-RES-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="9" t="str">
         <x:v>FS-REG-001</x:v>
       </x:c>
@@ -7241,10 +7244,10 @@
         <x:v>Register Read</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>REQ-FUNC-015~017; REQ-IF-006,REQ-IF-012</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-015~017; REQ-IF-004, REQ-IF-006, REQ-IF-012; REQ-ERR-002; REQ-REL-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="9" t="str">
         <x:v>FS-REG-002</x:v>
       </x:c>
@@ -7252,10 +7255,10 @@
         <x:v>Register Write Transaction</x:v>
       </x:c>
       <x:c r="C21" s="9" t="str">
-        <x:v>REQ-FUNC-016~018; REQ-IF-012; REQ-REL-002~003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-016~018; REQ-IF-004, REQ-IF-006, REQ-IF-012; REQ-ERR-002; REQ-REL-002~003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="9" t="str">
         <x:v>FS-REG-003</x:v>
       </x:c>
@@ -7263,10 +7266,10 @@
         <x:v>Device Reset</x:v>
       </x:c>
       <x:c r="C22" s="9" t="str">
-        <x:v>REQ-FUNC-019</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-019; REQ-IF-004; REQ-ERR-002; REQ-REL-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="9" t="str">
         <x:v>FS-SIG-001</x:v>
       </x:c>
@@ -7274,10 +7277,10 @@
         <x:v>Signal Map 구성</x:v>
       </x:c>
       <x:c r="C23" s="9" t="str">
-        <x:v>REQ-FUNC-020,REQ-FUNC-023~026; REQ-DATA-009~010</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-020, REQ-FUNC-023~026; REQ-DATA-009~010</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="9" t="str">
         <x:v>FS-SIG-002</x:v>
       </x:c>
@@ -7285,10 +7288,10 @@
         <x:v>Signal 물리값 Read</x:v>
       </x:c>
       <x:c r="C24" s="9" t="str">
-        <x:v>REQ-FUNC-020~025,REQ-FUNC-028~029; REQ-IF-013</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-020~025, REQ-FUNC-028~029; REQ-IF-004, REQ-IF-006, REQ-IF-013; REQ-ERR-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="9" t="str">
         <x:v>FS-SIG-003</x:v>
       </x:c>
@@ -7296,10 +7299,10 @@
         <x:v>Signal 물리값 Write</x:v>
       </x:c>
       <x:c r="C25" s="9" t="str">
-        <x:v>REQ-FUNC-020~025,REQ-FUNC-028~029; REQ-IF-013</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-020~025, REQ-FUNC-028~029; REQ-IF-004, REQ-IF-013; REQ-ERR-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="9" t="str">
         <x:v>FS-SIG-004</x:v>
       </x:c>
@@ -7307,10 +7310,10 @@
         <x:v>Init Image 합성</x:v>
       </x:c>
       <x:c r="C26" s="9" t="str">
-        <x:v>REQ-FUNC-021~028; REQ-FUNC-012</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-021~025, REQ-FUNC-027~028; REQ-ERR-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="9" t="str">
         <x:v>FS-MON-001</x:v>
       </x:c>
@@ -7318,10 +7321,10 @@
         <x:v>Monitoring Start/Stop</x:v>
       </x:c>
       <x:c r="C27" s="9" t="str">
-        <x:v>REQ-FUNC-030,REQ-FUNC-032,REQ-FUNC-039</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-030, REQ-FUNC-032, REQ-FUNC-039; REQ-IF-004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="9" t="str">
         <x:v>FS-MON-002</x:v>
       </x:c>
@@ -7329,10 +7332,10 @@
         <x:v>ReadOption Candidate 적용</x:v>
       </x:c>
       <x:c r="C28" s="9" t="str">
-        <x:v>REQ-FUNC-031,REQ-FUNC-038; REQ-PERF-004</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-031, REQ-FUNC-038; REQ-IF-004; REQ-PERF-004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="9" t="str">
         <x:v>FS-MON-003</x:v>
       </x:c>
@@ -7340,10 +7343,10 @@
         <x:v>Periodic Snapshot 생성</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
-        <x:v>REQ-FUNC-032~033; REQ-IF-007,REQ-IF-014</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-032~033; REQ-COM-021; REQ-IF-004, REQ-IF-006~007, REQ-IF-014; REQ-PERF-002~003; REQ-REL-005; REQ-RES-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A30" s="9" t="str">
         <x:v>FS-MON-004</x:v>
       </x:c>
@@ -7351,10 +7354,10 @@
         <x:v>Change Snapshot Queue</x:v>
       </x:c>
       <x:c r="C30" s="9" t="str">
-        <x:v>REQ-FUNC-018,REQ-FUNC-034~035,REQ-FUNC-039; REQ-IF-014</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-018, REQ-FUNC-034~035, REQ-FUNC-039; REQ-COM-021; REQ-IF-004, REQ-IF-006~007, REQ-IF-014; REQ-PERF-002~003; REQ-REL-002, REQ-REL-004~006; REQ-RES-003~004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="9" t="str">
         <x:v>FS-MON-005</x:v>
       </x:c>
@@ -7365,7 +7368,7 @@
         <x:v>REQ-COM-016~021; REQ-IF-007</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="32" customHeight="1">
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="9" t="str">
         <x:v>FS-MON-006</x:v>
       </x:c>
@@ -7373,10 +7376,10 @@
         <x:v>10ms Output Pump</x:v>
       </x:c>
       <x:c r="C32" s="9" t="str">
-        <x:v>REQ-FUNC-036~038; REQ-PERF-002,REQ-PERF-004; REQ-DIAG-003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-033, REQ-FUNC-036~038; REQ-PERF-002, REQ-PERF-004; REQ-REL-006; REQ-DIAG-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="9" t="str">
         <x:v>FS-UI-001</x:v>
       </x:c>
@@ -7384,10 +7387,10 @@
         <x:v>Manual Read 및 Auto Read</x:v>
       </x:c>
       <x:c r="C33" s="9" t="str">
-        <x:v>REQ-FUNC-041,REQ-FUNC-043</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-040~041, REQ-FUNC-043</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="9" t="str">
         <x:v>FS-UI-002</x:v>
       </x:c>
@@ -7395,10 +7398,10 @@
         <x:v>Manual Write</x:v>
       </x:c>
       <x:c r="C34" s="9" t="str">
-        <x:v>REQ-FUNC-042</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-040, REQ-FUNC-042</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="9" t="str">
         <x:v>FS-UI-003</x:v>
       </x:c>
@@ -7406,10 +7409,10 @@
         <x:v>Signal Panel Control</x:v>
       </x:c>
       <x:c r="C35" s="9" t="str">
-        <x:v>REQ-FUNC-044</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-040, REQ-FUNC-044</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="9" t="str">
         <x:v>FS-DIAG-001</x:v>
       </x:c>
@@ -7417,10 +7420,10 @@
         <x:v>동기 오류 조회</x:v>
       </x:c>
       <x:c r="C36" s="9" t="str">
-        <x:v>REQ-ERR-004~006; REQ-DIAG-001,REQ-DIAG-004; REQ-IF-009~010</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="32" customHeight="1">
+        <x:v>REQ-IF-004~005, REQ-IF-009~010; REQ-ERR-004~006; REQ-DIAG-001; REQ-COMP-006; REQ-SEC-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A37" s="9" t="str">
         <x:v>FS-DIAG-002</x:v>
       </x:c>
@@ -7428,10 +7431,10 @@
         <x:v>비동기 Error Event 및 Stats</x:v>
       </x:c>
       <x:c r="C37" s="9" t="str">
-        <x:v>REQ-ERR-006~008; REQ-DIAG-002~005; REQ-RES-003~004</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="32" customHeight="1">
+        <x:v>REQ-FUNC-035; REQ-IF-004, REQ-IF-009, REQ-IF-011; REQ-ERR-001, REQ-ERR-004~007; REQ-REL-002, REQ-REL-004; REQ-RES-003~004; REQ-DIAG-002~005; REQ-COMP-006</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="9" t="str">
         <x:v>FS-SHUT-001</x:v>
       </x:c>
@@ -7439,13 +7442,13 @@
         <x:v>측정 종료 Finalize</x:v>
       </x:c>
       <x:c r="C38" s="9" t="str">
-        <x:v>REQ-FUNC-008; REQ-PERF-006; REQ-RES-002</x:v>
+        <x:v>REQ-FUNC-008; REQ-PERF-006; REQ-REL-003; REQ-RES-002</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbee46007bb24344"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd58cff352904931"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7454,12 +7457,12 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="88" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="62.130001068115234" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A1" s="21" t="str">
         <x:v>Design Component ID</x:v>
       </x:c>
@@ -7470,7 +7473,7 @@
         <x:v>Responsibility</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="32" customHeight="1">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="9" t="str">
         <x:v>DC-01</x:v>
       </x:c>
@@ -7481,7 +7484,7 @@
         <x:v>CAPL_DLL_INFO4, __stdcall, Context Handle, Length/Capacity 검증, 21개 Export</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="32" customHeight="1">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="9" t="str">
         <x:v>DC-02</x:v>
       </x:c>
@@ -7492,7 +7495,7 @@
         <x:v>단일 활성 Context의 상태·Configuration·서비스·Queue 소유</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="32" customHeight="1">
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="9" t="str">
         <x:v>DC-03</x:v>
       </x:c>
@@ -7503,7 +7506,7 @@
         <x:v>Refresh/Connect/Disconnect/Finalize, 상태·Generation, 자동 재연결</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="32" customHeight="1">
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="9" t="str">
         <x:v>DC-04</x:v>
       </x:c>
@@ -7514,7 +7517,7 @@
         <x:v>UTF-8 CSV Parsing, 교차 검증, 임시 Configuration 및 원자 승격</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="32" customHeight="1">
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="9" t="str">
         <x:v>DC-05</x:v>
       </x:c>
@@ -7525,7 +7528,7 @@
         <x:v>Index/PortSlot/Slave_ID O(1) 조회와 Device Runtime 소유</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="32" customHeight="1">
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="9" t="str">
         <x:v>DC-06</x:v>
       </x:c>
@@ -7536,7 +7539,7 @@
         <x:v>공유 Register, 권한 Bitmap, 원자 Read/Write/Reset</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="32" customHeight="1">
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="9" t="str">
         <x:v>DC-07</x:v>
       </x:c>
@@ -7547,7 +7550,7 @@
         <x:v>Frame/Bit/Endian/Type/Scale/Offset/Init 변환</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="32" customHeight="1">
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="9" t="str">
         <x:v>DC-08</x:v>
       </x:c>
@@ -7558,7 +7561,7 @@
         <x:v>Frame 검증, CRC, FC03/04/10, Exception Response</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="32" customHeight="1">
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="9" t="str">
         <x:v>DC-09</x:v>
       </x:c>
@@ -7569,7 +7572,7 @@
         <x:v>Overlapped COM I/O, DCB, Cancel I/O, OS 오류 캡처</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="32" customHeight="1">
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="9" t="str">
         <x:v>DC-10</x:v>
       </x:c>
@@ -7580,7 +7583,7 @@
         <x:v>Port 단독 소유, t1.5/t3.5 조립, 순차 요청 처리</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="32" customHeight="1">
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="9" t="str">
         <x:v>DC-11</x:v>
       </x:c>
@@ -7591,7 +7594,7 @@
         <x:v>Periodic Snapshot, Port별 Change FIFO, Sequence/Stats</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="32" customHeight="1">
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="9" t="str">
         <x:v>DC-12</x:v>
       </x:c>
@@ -7602,7 +7605,7 @@
         <x:v>LastSyncError, Error Event FIFO, Counter/Latch</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="32" customHeight="1">
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="9" t="str">
         <x:v>DC-13</x:v>
       </x:c>
@@ -7613,7 +7616,7 @@
         <x:v>Context·경로·Buffer 은닉, Lifecycle Polling, 공통 오류 출력</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="32" customHeight="1">
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="9" t="str">
         <x:v>DC-14</x:v>
       </x:c>
@@ -7624,7 +7627,7 @@
         <x:v>ReadOption, 1,000ms Cycle, 10ms Pump, CAN Frame 생성</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="32" customHeight="1">
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="9" t="str">
         <x:v>DC-15</x:v>
       </x:c>
@@ -7635,7 +7638,7 @@
         <x:v>Connect/ReadSwitch, Manual Read/Write, Signal System Variable Adapter</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="32" customHeight="1">
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="9" t="str">
         <x:v>DC-16</x:v>
       </x:c>
@@ -7644,12 +7647,23 @@
       </x:c>
       <x:c r="C17" s="9" t="str">
         <x:v>오류 코드·공개 상수의 C++/CAPL 단일 기준 생성 및 검증</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" t="str">
+        <x:v>DC-17</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>Build &amp; Packaging</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="str">
+        <x:v>Win32/x86 빌드, Vector SDK 경로 주입, 배포 패키지 구조 및 후속 x64 경계 관리</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07fd9de29e91449d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84bc3bf431b74820"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7732,7 +7746,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdae6a788e5384210"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R599cce7077cf45ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
검증: Phase 1 CAPL DLL ABI 보완
생산 DLL의 21개 공개 API를 유지하면서 시험 전용 CAPL ABI Fixture를 추가했습니다.
Context 수명주기, 배열 및 F[1] 왕복, Capacity와 출력 불변성 검증을 강화했습니다.
요구사양서, 기능사양서, 개발설계서와 Traceability Matrix에 검증 결과를 반영했습니다.
</commit_message>
<xml_diff>
--- a/docs/04_Traceability/Modbus485Emulator_Traceability_Matrix.xlsx
+++ b/docs/04_Traceability/Modbus485Emulator_Traceability_Matrix.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R2b9ecc2e232c4856"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="2" r:id="R2ce999600d0f4252"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R59c595e390414e66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional Specs" sheetId="4" r:id="R3415fec85e8f41ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Components" sheetId="5" r:id="Re2d75cebc01843d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification Inputs" sheetId="6" r:id="Rce6cbd40336845a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R0c861755561543e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="2" r:id="Rb1f59e8001fd474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Radf4a759b93540cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional Specs" sheetId="4" r:id="R14fdc9525e104b18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Components" sheetId="5" r:id="Rb1202302cdb54ca8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification Inputs" sheetId="6" r:id="Ra3799b4c9b584386"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Verification" sheetId="7" r:id="Rb31731da52304c89"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +19,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="6">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -51,8 +52,32 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F4E78"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF375623"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -89,8 +114,23 @@
         <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="4">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -106,11 +146,39 @@
         <x:color rgb="FFB7C9D6"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="43">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -177,6 +245,46 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -818,11 +926,13 @@
         <x:v>DC-01 CAPL ABI Adapter; DC-02 EmulatorContext</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>CANalyzer 9.x x86 DLL 로딩 및 중복 Context 시험</x:v>
-      </x:c>
-      <x:c r="F2" s="23" t="str"/>
+        <x:v>Context 초기화·중복·잘못된 Handle·Finalize 후 호출·재초기화 자동 시험과 CANalyzer 9.x 실행</x:v>
+      </x:c>
+      <x:c r="F2" s="23" t="str">
+        <x:v>TC-P1-AUTO-002; TC-P1-ENV-001</x:v>
+      </x:c>
       <x:c r="G2" s="24" t="str">
-        <x:v>Defined</x:v>
+        <x:v>Phase 1 자동 검증 PASS / CANalyzer 9.x 대기</x:v>
       </x:c>
       <x:c r="H2" s="9" t="str">
         <x:v>FR-LIFE-009,016; IF-CTX-001~003,007</x:v>
@@ -2714,11 +2824,13 @@
         <x:v>DC-01 CAPL ABI Adapter</x:v>
       </x:c>
       <x:c r="E81" s="9" t="str">
-        <x:v>Vector Sample 기반 x86 최소 ABI 시험</x:v>
-      </x:c>
-      <x:c r="F81" s="23" t="str"/>
+        <x:v>Win32/x86 DLL Load, caplDllTable4, __stdcall Export와 CAPL compile/runtime 시험</x:v>
+      </x:c>
+      <x:c r="F81" s="23" t="str">
+        <x:v>TC-P1-AUTO-001; TC-P1-CAPL-001; TC-P1-ENV-001</x:v>
+      </x:c>
       <x:c r="G81" s="24" t="str">
-        <x:v>Defined</x:v>
+        <x:v>Phase 1 자동 검증 PASS / CANalyzer 9.x 대기</x:v>
       </x:c>
       <x:c r="H81" s="9" t="str">
         <x:v>FACT-DLL-001~005; IF-ABI-009</x:v>
@@ -2740,9 +2852,11 @@
       <x:c r="E82" s="9" t="str">
         <x:v>Export Table 이름·Wrapper 호출 시험</x:v>
       </x:c>
-      <x:c r="F82" s="23" t="str"/>
+      <x:c r="F82" s="23" t="str">
+        <x:v>TC-P1-AUTO-001; TC-P1-CAPL-001; TC-P1-ENV-001</x:v>
+      </x:c>
       <x:c r="G82" s="24" t="str">
-        <x:v>Defined</x:v>
+        <x:v>Phase 1 자동 검증 PASS / CANalyzer 9.x 대기</x:v>
       </x:c>
       <x:c r="H82" s="9" t="str">
         <x:v>IF-NAME-001~003; IF-CTX-001~006</x:v>
@@ -2753,7 +2867,7 @@
         <x:v>REQ-IF-003</x:v>
       </x:c>
       <x:c r="B83" s="9" t="str">
-        <x:v>DLL 경계에는 32bit long 상태, Scalar, 숫자 Reference 및 1차원 char[]/word[]/long[]만 사용하고 사용자 struct와 C++ 객체를 노출하지 않아야 한다.</x:v>
+        <x:v>DLL 경계에는 32bit long 상태, Scalar 및 1차원 char[]/word[]/long[]만 사용하고 Signal 물리값 출력은 저수준 ABI에서 1요소 F[]로 전달해야 하며 사용자 struct와 C++ 객체를 노출하지 않아야 한다.</x:v>
       </x:c>
       <x:c r="C83" s="9" t="str">
         <x:v>FS-INIT-001</x:v>
@@ -2762,11 +2876,13 @@
         <x:v>DC-01 CAPL ABI Adapter</x:v>
       </x:c>
       <x:c r="E83" s="9" t="str">
-        <x:v>최소 ABI Probe 및 Buffer 불변 시험</x:v>
-      </x:c>
-      <x:c r="F83" s="23" t="str"/>
+        <x:v>생산 Table 메타데이터와 별도 ABI Fixture의 char[]/word[]/long[]/F[1] 성공 왕복 및 Buffer 불변 시험</x:v>
+      </x:c>
+      <x:c r="F83" s="23" t="str">
+        <x:v>TC-P1-AUTO-004; TC-P1-CAPL-001; TC-P1-ENV-001</x:v>
+      </x:c>
       <x:c r="G83" s="24" t="str">
-        <x:v>Defined</x:v>
+        <x:v>Phase 1 자동 검증 PASS / CANalyzer 9.x 대기</x:v>
       </x:c>
       <x:c r="H83" s="9" t="str">
         <x:v>IF-ABI-001~011</x:v>
@@ -2788,9 +2904,11 @@
       <x:c r="E84" s="9" t="str">
         <x:v>21개 Export Table/Wrapper Contract 시험</x:v>
       </x:c>
-      <x:c r="F84" s="23" t="str"/>
+      <x:c r="F84" s="23" t="str">
+        <x:v>TC-P1-AUTO-001; TC-P1-CAPL-001; TC-P1-ENV-001</x:v>
+      </x:c>
       <x:c r="G84" s="24" t="str">
-        <x:v>Defined</x:v>
+        <x:v>Phase 1 자동 검증 PASS / CANalyzer 9.x 대기</x:v>
       </x:c>
       <x:c r="H84" s="9" t="str">
         <x:v>IF-API-001~021</x:v>
@@ -2812,9 +2930,11 @@
       <x:c r="E85" s="9" t="str">
         <x:v>동기/비동기/No Data 반환 시험</x:v>
       </x:c>
-      <x:c r="F85" s="23" t="str"/>
+      <x:c r="F85" s="23" t="str">
+        <x:v>TC-P1-AUTO-002; TC-P1-AUTO-003; TC-P1-ENV-001</x:v>
+      </x:c>
       <x:c r="G85" s="24" t="str">
-        <x:v>Defined</x:v>
+        <x:v>Phase 1 자동 검증 PASS / CANalyzer 9.x 대기</x:v>
       </x:c>
       <x:c r="H85" s="9" t="str">
         <x:v>IF-RET-001~009; IF-CODE-001~004</x:v>
@@ -2836,9 +2956,11 @@
       <x:c r="E86" s="9" t="str">
         <x:v>Buffer 부족·Embedded NUL·실패 시 출력 유지 시험</x:v>
       </x:c>
-      <x:c r="F86" s="23" t="str"/>
+      <x:c r="F86" s="23" t="str">
+        <x:v>TC-P1-AUTO-003; TC-P1-CAPL-001; TC-P1-ENV-001</x:v>
+      </x:c>
       <x:c r="G86" s="24" t="str">
-        <x:v>Defined</x:v>
+        <x:v>Phase 1 자동 검증 PASS / CANalyzer 9.x 대기</x:v>
       </x:c>
       <x:c r="H86" s="9" t="str">
         <x:v>IF-ABI-006~007,010~011; IF-RET-002~007</x:v>
@@ -2980,9 +3102,11 @@
       <x:c r="E92" s="9" t="str">
         <x:v>Quantity/Capacity 조합 및 실패 불변 시험</x:v>
       </x:c>
-      <x:c r="F92" s="23" t="str"/>
+      <x:c r="F92" s="23" t="str">
+        <x:v>TC-P1-AUTO-003; TC-P1-AUTO-004</x:v>
+      </x:c>
       <x:c r="G92" s="24" t="str">
-        <x:v>Defined</x:v>
+        <x:v>Phase 1 자동 검증 PASS</x:v>
       </x:c>
       <x:c r="H92" s="9" t="str">
         <x:v>IF-REG-001~012</x:v>
@@ -2993,7 +3117,7 @@
         <x:v>REQ-IF-013</x:v>
       </x:c>
       <x:c r="B93" s="9" t="str">
-        <x:v>ReadSignal은 성공 시에만 OutPhysicalValue를 갱신하고 WriteSignal은 Index, SignalName, double 물리값을 사용해야 한다.</x:v>
+        <x:v>ReadSignal은 성공 시에만 저수준 OutPhysicalValue[0]을 갱신하고 CAPL Core는 이를 double&amp; 출력으로 감싸야 하며, WriteSignal은 Index, SignalName, double 물리값을 사용해야 한다.</x:v>
       </x:c>
       <x:c r="C93" s="9" t="str">
         <x:v>FS-SIG-002,FS-SIG-003</x:v>
@@ -3002,11 +3126,13 @@
         <x:v>DC-01 CAPL ABI Adapter; DC-07 SignalCodec</x:v>
       </x:c>
       <x:c r="E93" s="9" t="str">
-        <x:v>정상/오류 시 Reference copy-restore 시험</x:v>
-      </x:c>
-      <x:c r="F93" s="23" t="str"/>
+        <x:v>F[1] 출력 실패 불변성과 시험 Fixture 성공 왕복, CANalyzer x86 호출 시험</x:v>
+      </x:c>
+      <x:c r="F93" s="23" t="str">
+        <x:v>TC-P1-AUTO-003; TC-P1-AUTO-004; TC-P1-ENV-001</x:v>
+      </x:c>
       <x:c r="G93" s="24" t="str">
-        <x:v>Defined</x:v>
+        <x:v>Phase 1 자동 검증 PASS / CANalyzer 9.x 대기</x:v>
       </x:c>
       <x:c r="H93" s="9" t="str">
         <x:v>IF-SIG-001~007</x:v>
@@ -3748,9 +3874,11 @@
       <x:c r="E124" s="9" t="str">
         <x:v>깨끗한 PC Win32 Build 및 CANalyzer 로딩 시험</x:v>
       </x:c>
-      <x:c r="F124" s="23" t="str"/>
+      <x:c r="F124" s="23" t="str">
+        <x:v>TC-P1-AUTO-001; TC-P1-ENV-001</x:v>
+      </x:c>
       <x:c r="G124" s="24" t="str">
-        <x:v>Defined</x:v>
+        <x:v>Phase 1 자동 검증 PASS / CANalyzer 9.x 대기</x:v>
       </x:c>
       <x:c r="H124" s="9" t="str">
         <x:v>ENV-001~002,010~011; COMP-001~002,008</x:v>
@@ -3772,9 +3900,11 @@
       <x:c r="E125" s="9" t="str">
         <x:v>설치 경로 변경·Clean Build 시험</x:v>
       </x:c>
-      <x:c r="F125" s="23" t="str"/>
+      <x:c r="F125" s="23" t="str">
+        <x:v>TC-P1-AUTO-001</x:v>
+      </x:c>
       <x:c r="G125" s="24" t="str">
-        <x:v>Defined</x:v>
+        <x:v>Phase 1 자동 검증 PASS</x:v>
       </x:c>
       <x:c r="H125" s="9" t="str">
         <x:v>DES-BUILD-001~005; TBD-059</x:v>
@@ -3796,9 +3926,11 @@
       <x:c r="E126" s="9" t="str">
         <x:v>공개 Export/문서에 Legacy 이름 부재 검토</x:v>
       </x:c>
-      <x:c r="F126" s="23" t="str"/>
+      <x:c r="F126" s="23" t="str">
+        <x:v>TC-P1-AUTO-001</x:v>
+      </x:c>
       <x:c r="G126" s="24" t="str">
-        <x:v>Defined</x:v>
+        <x:v>Phase 1 자동 검증 PASS</x:v>
       </x:c>
       <x:c r="H126" s="9" t="str">
         <x:v>PRJ-005~006; COMP-009~010</x:v>
@@ -3820,9 +3952,11 @@
       <x:c r="E127" s="9" t="str">
         <x:v>Win32 타입 크기 검토; x64는 후속 체크리스트</x:v>
       </x:c>
-      <x:c r="F127" s="23" t="str"/>
+      <x:c r="F127" s="23" t="str">
+        <x:v>TC-P1-AUTO-001</x:v>
+      </x:c>
       <x:c r="G127" s="24" t="str">
-        <x:v>Defined</x:v>
+        <x:v>Phase 1 자동 검증 PASS</x:v>
       </x:c>
       <x:c r="H127" s="9" t="str">
         <x:v>ENV-011; FUT-001~005</x:v>
@@ -3956,7 +4090,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R225405ba02354d1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R514d4d82acc94649"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7013,7 +7147,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R100a34472a584bbc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcaad5af6600346c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7448,7 +7582,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd58cff352904931"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4438aa5e2c6463b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7663,7 +7797,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84bc3bf431b74820"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e73861150a64c73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7693,10 +7827,10 @@
         <x:v>CANalyzer 9.x x86 ABI</x:v>
       </x:c>
       <x:c r="B2" s="25" t="str">
-        <x:v>검증 필요</x:v>
+        <x:v>자동 검증 PASS / CANalyzer 9.x 실환경 대기</x:v>
       </x:c>
       <x:c r="C2" s="25" t="str">
-        <x:v>Phase 1 minimum probe</x:v>
+        <x:v>생산 21 API + 시험 전용 ABI Fixture 자동 Probe 후 CANalyzer 9.x SP8 측정 실행</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="32" customHeight="1">
@@ -7746,7 +7880,164 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R599cce7077cf45ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5050e80d13e24eae"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="36" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="46" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="26" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="52" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="32" t="str">
+        <x:v>Test Case ID</x:v>
+      </x:c>
+      <x:c r="B1" s="32" t="str">
+        <x:v>검증 범위</x:v>
+      </x:c>
+      <x:c r="C1" s="32" t="str">
+        <x:v>실행 방법</x:v>
+      </x:c>
+      <x:c r="D1" s="32" t="str">
+        <x:v>환경</x:v>
+      </x:c>
+      <x:c r="E1" s="32" t="str">
+        <x:v>결과</x:v>
+      </x:c>
+      <x:c r="F1" s="32" t="str">
+        <x:v>비고</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A2" s="36" t="str">
+        <x:v>TC-P1-AUTO-001</x:v>
+      </x:c>
+      <x:c r="B2" s="35" t="str">
+        <x:v>Win32 빌드와 생산 CAPL Table 21 API</x:v>
+      </x:c>
+      <x:c r="C2" s="35" t="str">
+        <x:v>MSBuild Debug/Release, CMake Release, dumpbin 및 ABI 메타데이터 검사</x:v>
+      </x:c>
+      <x:c r="D2" s="35" t="str">
+        <x:v>Visual Studio 18 / Win32</x:v>
+      </x:c>
+      <x:c r="E2" s="39" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F2" s="35" t="str">
+        <x:v>x86(14C), 생산 API 정확히 21개, caplDllTable4 확인</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="36" t="str">
+        <x:v>TC-P1-AUTO-002</x:v>
+      </x:c>
+      <x:c r="B3" s="35" t="str">
+        <x:v>Context 수명주기</x:v>
+      </x:c>
+      <x:c r="C3" s="35" t="str">
+        <x:v>네이티브 M485E.AbiProbe</x:v>
+      </x:c>
+      <x:c r="D3" s="35" t="str">
+        <x:v>Win32</x:v>
+      </x:c>
+      <x:c r="E3" s="39" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F3" s="35" t="str">
+        <x:v>0 Handle, 중복, 잘못된 Handle, Finalize 후 호출, 재초기화</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A4" s="36" t="str">
+        <x:v>TC-P1-AUTO-003</x:v>
+      </x:c>
+      <x:c r="B4" s="35" t="str">
+        <x:v>Capacity·문자열 검증·출력 불변성</x:v>
+      </x:c>
+      <x:c r="C4" s="35" t="str">
+        <x:v>네이티브 M485E.AbiProbe</x:v>
+      </x:c>
+      <x:c r="D4" s="35" t="str">
+        <x:v>Win32</x:v>
+      </x:c>
+      <x:c r="E4" s="39" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F4" s="35" t="str">
+        <x:v>작은 Capacity, Embedded NUL, 길이 불일치, 실패 시 caller-owned 출력 보존</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="36" t="str">
+        <x:v>TC-P1-AUTO-004</x:v>
+      </x:c>
+      <x:c r="B5" s="35" t="str">
+        <x:v>char[]/word[]/long[]/F[1] 성공 왕복</x:v>
+      </x:c>
+      <x:c r="C5" s="35" t="str">
+        <x:v>시험 전용 M485E.CaplAbiFixture + 네이티브/CAPL Probe</x:v>
+      </x:c>
+      <x:c r="D5" s="35" t="str">
+        <x:v>Win32</x:v>
+      </x:c>
+      <x:c r="E5" s="39" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F5" s="35" t="str">
+        <x:v>시험 Fixture는 생산 21 API와 분리</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="36" t="str">
+        <x:v>TC-P1-CAPL-001</x:v>
+      </x:c>
+      <x:c r="B6" s="35" t="str">
+        <x:v>CAPL 소스 컴파일</x:v>
+      </x:c>
+      <x:c r="C6" s="35" t="str">
+        <x:v>CANalyzer 13 Exec32 caplcompexec</x:v>
+      </x:c>
+      <x:c r="D6" s="35" t="str">
+        <x:v>CANalyzer 13 x86 compiler</x:v>
+      </x:c>
+      <x:c r="E6" s="39" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F6" s="35" t="str">
+        <x:v>컴파일만 확인, Measurement 실행 아님</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="36" t="str">
+        <x:v>TC-P1-ENV-001</x:v>
+      </x:c>
+      <x:c r="B7" s="35" t="str">
+        <x:v>CANalyzer 9.x SP8 실제 로드·호출·측정</x:v>
+      </x:c>
+      <x:c r="C7" s="35" t="str">
+        <x:v>M485E_Phase1_AbiProbe.can Measurement 실행</x:v>
+      </x:c>
+      <x:c r="D7" s="35" t="str">
+        <x:v>회사 CANalyzer 9.x SP8 x86</x:v>
+      </x:c>
+      <x:c r="E7" s="42" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="F7" s="35" t="str">
+        <x:v>실환경 결과를 임의로 PASS 처리하지 않음</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
릴리스: Modbus485Emulator v0.5.0 구현 및 배포 준비
</commit_message>
<xml_diff>
--- a/docs/04_Traceability/Modbus485Emulator_Traceability_Matrix.xlsx
+++ b/docs/04_Traceability/Modbus485Emulator_Traceability_Matrix.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R593d0f1a409c4bd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="2" r:id="Ra94327c87b364616"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rdb7ae70dc0064db8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional Specs" sheetId="4" r:id="R89bbcf80e9e34612"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Components" sheetId="5" r:id="R3f8fd0682bcc4c81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification Inputs" sheetId="6" r:id="R063d534d39484d74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Verification" sheetId="7" r:id="R0adc9d1fbc374ad3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Verification" sheetId="8" r:id="R3c1465886ef44bf0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3-10 Verification" sheetId="9" r:id="R544e77aa1feb4397"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v0.3.0 Traceability" sheetId="10" r:id="R5076e0f5e9704c40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R9869f5ea61a442e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="2" r:id="R4ee31e3544f642d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rbd19b3ee850444ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional Specs" sheetId="4" r:id="Rbb215e9051664201"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Components" sheetId="5" r:id="R6528b4b8ab9e4d69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification Inputs" sheetId="6" r:id="R4a88a93129ed4034"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Verification" sheetId="7" r:id="R34fdfe7f134a4029"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Verification" sheetId="8" r:id="R1eb5e5a782dd4a30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3-10 Verification" sheetId="9" r:id="R07d6a19c9c1a44b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v0.3.0 Traceability" sheetId="10" r:id="Rdb5d9cf260854225"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -86,7 +86,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="72">
+  <x:fills count="75">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -443,6 +443,21 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="6">
     <x:border/>
@@ -520,7 +535,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="196">
+  <x:cellXfs count="206">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1023,6 +1038,30 @@
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="71" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="72" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="73" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="72" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="74" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="73" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="73" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="73" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="74" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1443,7 +1482,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>0.4.0</x:v>
+        <x:v>0.5.0</x:v>
       </x:c>
       <x:c r="D7" s="11" t="str">
         <x:v>Requirements with Design</x:v>
@@ -1473,7 +1512,7 @@
         <x:v>Baseline Date</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-08-13</x:v>
+        <x:v>2026-08-17</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
         <x:v>Test Case IDs</x:v>
@@ -1630,25 +1669,25 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="187" t="str">
+      <x:c r="A1" s="197" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="B1" s="187" t="str">
+      <x:c r="B1" s="197" t="str">
         <x:v>Functional Specification</x:v>
       </x:c>
-      <x:c r="C1" s="187" t="str">
+      <x:c r="C1" s="197" t="str">
         <x:v>Design</x:v>
       </x:c>
-      <x:c r="D1" s="187" t="str">
+      <x:c r="D1" s="197" t="str">
         <x:v>Implementation</x:v>
       </x:c>
-      <x:c r="E1" s="187" t="str">
+      <x:c r="E1" s="197" t="str">
         <x:v>Automated Verification</x:v>
       </x:c>
-      <x:c r="F1" s="187" t="str">
+      <x:c r="F1" s="197" t="str">
         <x:v>External Verification</x:v>
       </x:c>
-      <x:c r="G1" s="187" t="str">
+      <x:c r="G1" s="197" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -1671,7 +1710,7 @@
       <x:c r="F2" s="63" t="str">
         <x:v>EV-017</x:v>
       </x:c>
-      <x:c r="G2" s="189" t="str">
+      <x:c r="G2" s="199" t="str">
         <x:v>Auto PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -1694,7 +1733,7 @@
       <x:c r="F3" s="63" t="str">
         <x:v>EV-017</x:v>
       </x:c>
-      <x:c r="G3" s="189" t="str">
+      <x:c r="G3" s="199" t="str">
         <x:v>Auto PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -1717,7 +1756,7 @@
       <x:c r="F4" s="63" t="str">
         <x:v>EV-017</x:v>
       </x:c>
-      <x:c r="G4" s="189" t="str">
+      <x:c r="G4" s="199" t="str">
         <x:v>Static PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -1740,7 +1779,7 @@
       <x:c r="F5" s="63" t="str">
         <x:v>EV-018</x:v>
       </x:c>
-      <x:c r="G5" s="189" t="str">
+      <x:c r="G5" s="199" t="str">
         <x:v>Auto PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -1763,7 +1802,7 @@
       <x:c r="F6" s="63" t="str">
         <x:v>EV-018</x:v>
       </x:c>
-      <x:c r="G6" s="189" t="str">
+      <x:c r="G6" s="199" t="str">
         <x:v>Auto/Static PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -1786,7 +1825,7 @@
       <x:c r="F7" s="63" t="str">
         <x:v>EV-001</x:v>
       </x:c>
-      <x:c r="G7" s="189" t="str">
+      <x:c r="G7" s="199" t="str">
         <x:v>Auto PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -1809,7 +1848,7 @@
       <x:c r="F8" s="63" t="str">
         <x:v>EV-018</x:v>
       </x:c>
-      <x:c r="G8" s="189" t="str">
+      <x:c r="G8" s="199" t="str">
         <x:v>Auto/Static PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -1832,7 +1871,7 @@
       <x:c r="F9" s="63" t="str">
         <x:v>EV-017~EV-018</x:v>
       </x:c>
-      <x:c r="G9" s="189" t="str">
+      <x:c r="G9" s="199" t="str">
         <x:v>Auto PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -2666,19 +2705,19 @@
         <x:v>REQ-FUNC-031</x:v>
       </x:c>
       <x:c r="B32" s="9" t="str">
-        <x:v>ReadOption은 최대 200개 Rule의 0x80 Periodic 선택만 제어하고 여러 변경을 다음 1,000ms Cycle 경계에 원자 적용해야 한다.</x:v>
+        <x:v>ReadOption은 최대 200개 Rule의 0x80 Periodic 선택만 제어하고 다음 1,000ms Cycle 경계에 원자 적용해야 한다. Monitoring::Btn_ReadOption은 int32 Scalar 편의 버튼으로만 제공하며 별도 CAPL Handler 없이 기존 Check_ReadOption[200], 100ms Candidate 동기화와 Cycle 적용 정책을 유지해야 한다.</x:v>
       </x:c>
       <x:c r="C32" s="9" t="str">
-        <x:v>FS-MON-002</x:v>
+        <x:v>FS-MON-002; FS-UI-001</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str">
-        <x:v>DC-14 CAPL Monitoring</x:v>
+        <x:v>DC-14 CAPL Monitoring; DC-15 CAPL UI</x:v>
       </x:c>
       <x:c r="E32" s="9" t="str">
-        <x:v>다중 Checkbox 원자 적용·복원 시험</x:v>
+        <x:v>Btn_ReadOption int32 Scalar/no-handler, Check_ReadOption[200] 유지 및 Candidate/Applied 원자 적용 검사</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>TC-P9-STATIC-001; EV-008; EV-009; EV-010; EV-011</x:v>
+        <x:v>TC-P9-STATIC-001; TC-P10-STATIC-001; EV-011; EV-019</x:v>
       </x:c>
       <x:c r="G32" s="24" t="str">
         <x:v>부분 자동 검증 PASS / External Verification Pending</x:v>
@@ -5365,12 +5404,12 @@
         <x:v>FR-UI-016~018</x:v>
       </x:c>
     </x:row>
-    <x:row r="136" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="136" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A136" s="63" t="str">
         <x:v>REQ-FUNC-048</x:v>
       </x:c>
       <x:c r="B136" s="63" t="str">
-        <x:v>RTU 요청과 실제 응답 또는 무응답을 동일 Sequence의 REQ/RES 또는 REQ/NO_RES CSV 행으로 기록</x:v>
+        <x:v>RTU 요청과 실제 응답 또는 무응답을 동일 Sequence의 REQ/RES 또는 REQ/NO_RES CSV 행으로 빠짐없이 기록하고, 같은 Dequeue 문자열을 별도 Consumer 없이 최근 10줄 Panel 표시에 재사용</x:v>
       </x:c>
       <x:c r="C136" s="63" t="str">
         <x:v>FS-RTULOG-001</x:v>
@@ -5379,24 +5418,24 @@
         <x:v>DC-19 RTU Log Pipeline</x:v>
       </x:c>
       <x:c r="E136" s="63" t="str">
-        <x:v>Transaction pair·overflow·send result</x:v>
+        <x:v>Transaction pair·overflow·send result·single drain panel reuse</x:v>
       </x:c>
       <x:c r="F136" s="63" t="str">
-        <x:v>TC-V03-AUTO-001; EV-018</x:v>
+        <x:v>TC-V03-AUTO-001; TC-P10-STATIC-001; EV-018~019</x:v>
       </x:c>
       <x:c r="G136" s="63" t="str">
-        <x:v>Automated PASS / External Pending</x:v>
+        <x:v>Automated/Static PASS / External Pending</x:v>
       </x:c>
       <x:c r="H136" s="63" t="str">
-        <x:v>LOG-018~024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="137" ht="39.599998474121094" hidden="0" customHeight="1">
+        <x:v>LOG-018~028</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A137" s="63" t="str">
         <x:v>REQ-FUNC-049</x:v>
       </x:c>
       <x:c r="B137" s="63" t="str">
-        <x:v>RTU Log 파일 Open 성공 후 Capture를 시작하고, OFF·종료 시 최대 2,000ms Idle 대기 후 완료 행을 배출</x:v>
+        <x:v>RTU Log 파일 Open 성공 후 Capture를 시작하고 OFF·종료 시 최대 2,000ms Idle 대기 후 완료 행을 배출한다. CAPL Output View는 설정 이름으로 최근 10줄을 200ms 이상 간격 Overwrite하며 실패가 CSV를 중단하지 않고 OFF 후 마지막 표시를 유지</x:v>
       </x:c>
       <x:c r="C137" s="63" t="str">
         <x:v>FS-RTULOG-001</x:v>
@@ -5405,16 +5444,16 @@
         <x:v>DC-19 RTU Log Pipeline</x:v>
       </x:c>
       <x:c r="E137" s="63" t="str">
-        <x:v>Open-before-capture·2,000ms idle wait·drain</x:v>
+        <x:v>Open-before-capture·2,000ms idle wait·drain·최근10줄/200ms Output View</x:v>
       </x:c>
       <x:c r="F137" s="63" t="str">
-        <x:v>TC-V03-AUTO-001; TC-P9-STATIC-001; EV-018</x:v>
+        <x:v>TC-V03-AUTO-001; TC-P9-STATIC-001; TC-P10-STATIC-001; EV-018~019</x:v>
       </x:c>
       <x:c r="G137" s="63" t="str">
         <x:v>Automated/Static PASS / External Pending</x:v>
       </x:c>
       <x:c r="H137" s="63" t="str">
-        <x:v>FR-UI-021; LOG-022~024; ERR-044</x:v>
+        <x:v>FR-UI-021~023; LOG-022~028; ERR-044</x:v>
       </x:c>
     </x:row>
     <x:row r="138" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -5422,7 +5461,7 @@
         <x:v>REQ-IF-015</x:v>
       </x:c>
       <x:c r="B138" s="63" t="str">
-        <x:v>CAPL DLL Export Table은 Appendix A의 v0.4.0 23개 Entry를 정확히 제공하고 제거된 Monitoring·Change Queue API를 공개하지 않는다</x:v>
+        <x:v>CAPL DLL Export Table은 Appendix A의 v0.5.0 23개 Entry를 정확히 제공하고 제거된 Monitoring·Change Queue API를 공개하지 않는다</x:v>
       </x:c>
       <x:c r="C138" s="63" t="str">
         <x:v>FS-INIT-001; FS-MON-003; FS-DEVICE-001; FS-RTULOG-001</x:v>
@@ -5477,7 +5516,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R850ab91f2a644e33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5c26bf976754e3b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6216,19 +6255,19 @@
         <x:v>Monitoring</x:v>
       </x:c>
       <x:c r="C32" s="9" t="str">
-        <x:v>ReadOption은 최대 200개 Rule의 0x80 Periodic 선택만 제어하고 여러 변경을 다음 1,000ms Cycle 경계에 원자 적용해야 한다.</x:v>
+        <x:v>ReadOption은 최대 200개 Rule의 0x80 Periodic 선택만 제어하고 다음 1,000ms Cycle 경계에 원자 적용해야 한다. Monitoring::Btn_ReadOption은 int32 Scalar 편의 버튼으로만 제공하며 별도 CAPL Handler 없이 기존 Check_ReadOption[200], 100ms Candidate 동기화와 Cycle 적용 정책을 유지해야 한다.</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str">
         <x:v>FR-CAN-020~027,047,057</x:v>
       </x:c>
       <x:c r="E32" s="9" t="str">
-        <x:v>FS-MON-002</x:v>
+        <x:v>FS-MON-002; FS-UI-001</x:v>
       </x:c>
       <x:c r="F32" s="9" t="str">
-        <x:v>CAPL Monitoring</x:v>
+        <x:v>CAPL Monitoring; CAPL UI</x:v>
       </x:c>
       <x:c r="G32" s="9" t="str">
-        <x:v>다중 Checkbox 원자 적용·복원 시험</x:v>
+        <x:v>Btn_ReadOption int32 Scalar/no-handler, Check_ReadOption[200] 유지 및 Candidate/Applied 원자 적용 검사</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="32" customHeight="1">
@@ -8600,7 +8639,7 @@
         <x:v>CAPL source contract와 EV-017</x:v>
       </x:c>
     </x:row>
-    <x:row r="136" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="136" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A136" s="63" t="str">
         <x:v>REQ-FUNC-048</x:v>
       </x:c>
@@ -8608,10 +8647,10 @@
         <x:v>Diagnostics</x:v>
       </x:c>
       <x:c r="C136" s="63" t="str">
-        <x:v>RTU 요청과 실제 응답 또는 무응답을 동일 Sequence의 REQ/RES 또는 REQ/NO_RES CSV 행으로 기록</x:v>
+        <x:v>RTU 요청과 실제 응답 또는 무응답을 동일 Sequence의 REQ/RES 또는 REQ/NO_RES CSV 행으로 빠짐없이 기록하고, 같은 Dequeue 문자열을 별도 Consumer 없이 최근 10줄 Panel 표시에 재사용</x:v>
       </x:c>
       <x:c r="D136" s="63" t="str">
-        <x:v>LOG-018~024</x:v>
+        <x:v>LOG-018~028</x:v>
       </x:c>
       <x:c r="E136" s="63" t="str">
         <x:v>FS-RTULOG-001</x:v>
@@ -8620,10 +8659,10 @@
         <x:v>DC-19</x:v>
       </x:c>
       <x:c r="G136" s="63" t="str">
-        <x:v>RtuLogQueue/PortWorker 자동 시험과 EV-018</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="137" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>RtuLogQueue/PortWorker 자동 시험, CAPL 단일 Consumer 정적 계약과 EV-018~019</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A137" s="63" t="str">
         <x:v>REQ-FUNC-049</x:v>
       </x:c>
@@ -8631,10 +8670,10 @@
         <x:v>Diagnostics</x:v>
       </x:c>
       <x:c r="C137" s="63" t="str">
-        <x:v>RTU Log 파일 Open 성공 후 Capture를 시작하고, OFF·종료 시 최대 2,000ms Idle 대기 후 완료 행을 배출</x:v>
+        <x:v>RTU Log 파일 Open 성공 후 Capture를 시작하고 OFF·종료 시 최대 2,000ms Idle 대기 후 완료 행을 배출한다. CAPL Output View는 설정 이름으로 최근 10줄을 200ms 이상 간격 Overwrite하며 실패가 CSV를 중단하지 않고 OFF 후 마지막 표시를 유지</x:v>
       </x:c>
       <x:c r="D137" s="63" t="str">
-        <x:v>FR-UI-021; LOG-022~024; ERR-044</x:v>
+        <x:v>FR-UI-021~023; LOG-022~028; ERR-044</x:v>
       </x:c>
       <x:c r="E137" s="63" t="str">
         <x:v>FS-RTULOG-001</x:v>
@@ -8643,7 +8682,7 @@
         <x:v>DC-19</x:v>
       </x:c>
       <x:c r="G137" s="63" t="str">
-        <x:v>Core/Integration/CAPL source contract와 EV-018</x:v>
+        <x:v>Core/Integration/CAPL source contract와 EV-018~019</x:v>
       </x:c>
     </x:row>
     <x:row r="138" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -8654,7 +8693,7 @@
         <x:v>API</x:v>
       </x:c>
       <x:c r="C138" s="63" t="str">
-        <x:v>CAPL DLL Export Table은 Appendix A의 v0.4.0 23개 Entry를 정확히 제공하고 제거된 Monitoring·Change Queue API를 공개하지 않는다</x:v>
+        <x:v>CAPL DLL Export Table은 Appendix A의 v0.5.0 23개 Entry를 정확히 제공하고 제거된 Monitoring·Change Queue API를 공개하지 않는다</x:v>
       </x:c>
       <x:c r="D138" s="63" t="str">
         <x:v>IF-API-001~008; IF-API-011; IF-API-014~027; COMP-009</x:v>
@@ -8695,7 +8734,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8467b2888f743c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a0611f3cc0146a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9154,7 +9193,7 @@
         <x:v>FS-RTULOG-001</x:v>
       </x:c>
       <x:c r="B41" s="63" t="str">
-        <x:v>RTU 요청·응답 CSV 기록</x:v>
+        <x:v>RTU 전체 CSV 및 최근 10줄 CAPL Output View</x:v>
       </x:c>
       <x:c r="C41" s="63" t="str">
         <x:v>REQ-FUNC-048~049; REQ-IF-015~016</x:v>
@@ -9163,7 +9202,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67be2c7f869f476c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R343186bef1974b68"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9350,7 +9389,7 @@
         <x:v>CAPL UI</x:v>
       </x:c>
       <x:c r="C16" s="9" t="str">
-        <x:v>Connect/ReadSwitch, Manual Write Data[122], Signal System Variable Adapter, Register Read UI 미제공, Error Queue Stats 변화기반 진단 출력</x:v>
+        <x:v>Connect/ReadSwitch, Btn_ReadOption int32 Scalar 편의 변수(no-handler), Manual Write Data[122], Signal System Variable Adapter, Register Read UI 미제공, Error Queue Stats 변화기반 진단 출력</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -9394,13 +9433,13 @@
         <x:v>RTU Log Pipeline</x:v>
       </x:c>
       <x:c r="C20" s="63" t="str">
-        <x:v>PortWorker 관측점, Transaction Queue, REQ/RES·NO_RES pairing과 CAPL-only CSV Writer</x:v>
+        <x:v>PortWorker 관측점, Transaction Queue, REQ/RES·NO_RES pairing, CAPL-only 전체 CSV Writer와 동일 Drain 문자열의 최근 10줄·200ms Output View</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51fb07d3bff146b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R941f46324778426f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9507,7 +9546,7 @@
         <x:v>External Test Result</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>18건 Not Tested</x:v>
+        <x:v>19건 Not Tested</x:v>
       </x:c>
       <x:c r="C9" t="str">
         <x:v>docs/05_Test/Modbus485Emulator_External_Test_Result.xlsx</x:v>
@@ -9538,7 +9577,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdddb4b30b6e74683"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bdaeff5f72c40fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9845,7 +9884,7 @@
       <x:c r="D7" s="35" t="str">
         <x:v>CANalyzer 13 x86</x:v>
       </x:c>
-      <x:c r="E7" s="186" t="str">
+      <x:c r="E7" s="196" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F7" s="35" t="str">
@@ -9891,25 +9930,25 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="187" t="str">
+      <x:c r="A1" s="197" t="str">
         <x:v>Test Case ID</x:v>
       </x:c>
-      <x:c r="B1" s="187" t="str">
+      <x:c r="B1" s="197" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="C1" s="187" t="str">
+      <x:c r="C1" s="197" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="D1" s="187" t="str">
+      <x:c r="D1" s="197" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="E1" s="187" t="str">
+      <x:c r="E1" s="197" t="str">
         <x:v>Method</x:v>
       </x:c>
-      <x:c r="F1" s="187" t="str">
+      <x:c r="F1" s="197" t="str">
         <x:v>Result</x:v>
       </x:c>
-      <x:c r="G1" s="187" t="str">
+      <x:c r="G1" s="197" t="str">
         <x:v>External Follow-up</x:v>
       </x:c>
     </x:row>
@@ -9929,7 +9968,7 @@
       <x:c r="E2" s="63" t="str">
         <x:v>M485E.Core.Tests</x:v>
       </x:c>
-      <x:c r="F2" s="188" t="str">
+      <x:c r="F2" s="198" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G2" s="63" t="str">
@@ -9952,7 +9991,7 @@
       <x:c r="E3" s="63" t="str">
         <x:v>M485E.Core.Tests</x:v>
       </x:c>
-      <x:c r="F3" s="188" t="str">
+      <x:c r="F3" s="198" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G3" s="63" t="str">
@@ -9975,7 +10014,7 @@
       <x:c r="E4" s="63" t="str">
         <x:v>M485E.Core.Tests</x:v>
       </x:c>
-      <x:c r="F4" s="188" t="str">
+      <x:c r="F4" s="198" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G4" s="63" t="str">
@@ -9998,7 +10037,7 @@
       <x:c r="E5" s="63" t="str">
         <x:v>M485E.Core.Tests</x:v>
       </x:c>
-      <x:c r="F5" s="188" t="str">
+      <x:c r="F5" s="198" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G5" s="63" t="str">
@@ -10021,7 +10060,7 @@
       <x:c r="E6" s="63" t="str">
         <x:v>M485E.Core.Tests + FakeSerialTransport</x:v>
       </x:c>
-      <x:c r="F6" s="188" t="str">
+      <x:c r="F6" s="198" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G6" s="63" t="str">
@@ -10044,7 +10083,7 @@
       <x:c r="E7" s="63" t="str">
         <x:v>M485E.IntegrationTests</x:v>
       </x:c>
-      <x:c r="F7" s="188" t="str">
+      <x:c r="F7" s="198" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G7" s="63" t="str">
@@ -10067,14 +10106,14 @@
       <x:c r="E8" s="63" t="str">
         <x:v>Test-M485ECaplSources.ps1 + CANalyzer 13 Exec32 caplcompexec</x:v>
       </x:c>
-      <x:c r="F8" s="188" t="str">
+      <x:c r="F8" s="198" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G8" s="63" t="str">
-        <x:v>EV-008~EV-011, EV-016</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="39.599998474121094" hidden="0" customHeight="1">
+        <x:v>EV-008~EV-011, EV-016, EV-019</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A9" s="63" t="str">
         <x:v>TC-P10-STATIC-001</x:v>
       </x:c>
@@ -10085,19 +10124,19 @@
         <x:v>Static</x:v>
       </x:c>
       <x:c r="D9" s="63" t="str">
-        <x:v>UI System Variable adapter, Manual Write Data[122], Signal Control, Register Read UI 부재 계약</x:v>
+        <x:v>UI System Variable adapter, Btn_ReadOption int32 Scalar/no-handler, Check_ReadOption[200] 유지, RTU Log 단일 Drain·최근 10줄·200ms putValueToControl, Manual Write Data[122], Signal Control, Register Read UI 부재 계약</x:v>
       </x:c>
       <x:c r="E9" s="63" t="str">
         <x:v>Test-M485ECaplSources.ps1; Main compile in configured CANalyzer project</x:v>
       </x:c>
-      <x:c r="F9" s="189" t="str">
+      <x:c r="F9" s="199" t="str">
         <x:v>Static PASS / External Pending</x:v>
       </x:c>
       <x:c r="G9" s="63" t="str">
-        <x:v>EV-011~EV-013, EV-016</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="66" hidden="0" customHeight="1">
+        <x:v>EV-011~EV-013, EV-016, EV-019</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A10" s="63" t="str">
         <x:v>TC-REG-AUTO-001</x:v>
       </x:c>
@@ -10108,16 +10147,16 @@
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="D10" s="63" t="str">
-        <x:v>Windows x86/x64 Debug/Release, /W4 /WX, ErrorCodes 91/PublicConstants 189, 23 API ABI, RuleDataMeta[9], RTU 로그 idle wait, 1/4 Port·5 Port 경계, 누락 PortSlot, contract/core/integration/CAPL probes</x:v>
+        <x:v>Windows x86/x64 Debug/Release, /W4 /WX, ErrorCodes 91/PublicConstants 189, 23 API ABI, RuleDataMeta[9], RTU 로그 idle wait·단일 Drain Panel adapter, 1/4 Port·5 Port 경계, 누락 PortSlot, contract/core/integration/CAPL probes</x:v>
       </x:c>
       <x:c r="E10" s="63" t="str">
         <x:v>MSBuild + CMake + CTest + CANalyzer 13 x86 CAPL compiler</x:v>
       </x:c>
-      <x:c r="F10" s="188" t="str">
+      <x:c r="F10" s="198" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G10" s="63" t="str">
-        <x:v>EV-001~EV-018</x:v>
+        <x:v>EV-001~EV-019</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -10136,16 +10175,16 @@
       <x:c r="E11" s="63" t="str">
         <x:v>M485E.Core.Tests + M485E.IntegrationTests + Test-M485ECaplSources.ps1</x:v>
       </x:c>
-      <x:c r="F11" s="189" t="str">
+      <x:c r="F11" s="199" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G11" s="63" t="str">
-        <x:v>EV-017~EV-018</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>EV-017~EV-019</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A12" s="63" t="str">
-        <x:v>EV-001~EV-018</x:v>
+        <x:v>EV-001~EV-019</x:v>
       </x:c>
       <x:c r="B12" s="63" t="str">
         <x:v>External</x:v>
@@ -10154,12 +10193,12 @@
         <x:v>External</x:v>
       </x:c>
       <x:c r="D12" s="63" t="str">
-        <x:v>CANalyzer 9.x/18, SystemBase Multi USB-485, Board, Panel, virtual CAN, RTU CSV</x:v>
+        <x:v>CANalyzer 9.x/18, SystemBase Multi USB-485, Board, Panel, CAPL Output View, virtual CAN, RTU CSV</x:v>
       </x:c>
       <x:c r="E12" s="63" t="str">
         <x:v>External Verification Guide</x:v>
       </x:c>
-      <x:c r="F12" s="188" t="str">
+      <x:c r="F12" s="198" t="str">
         <x:v>Not Tested</x:v>
       </x:c>
       <x:c r="G12" s="63" t="str">
@@ -10182,7 +10221,7 @@
       <x:c r="E13" s="63" t="str">
         <x:v>CANalyzer 13 Exec32 caplcompexec.exe</x:v>
       </x:c>
-      <x:c r="F13" s="188" t="str">
+      <x:c r="F13" s="198" t="str">
         <x:v>PASS (warning-free)</x:v>
       </x:c>
       <x:c r="G13" s="63" t="str">

</xml_diff>

<commit_message>
릴리스: Modbus485Emulator v0.6.0 Panel Generator 구현 및 배포 준비
</commit_message>
<xml_diff>
--- a/docs/04_Traceability/Modbus485Emulator_Traceability_Matrix.xlsx
+++ b/docs/04_Traceability/Modbus485Emulator_Traceability_Matrix.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R9869f5ea61a442e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="2" r:id="R4ee31e3544f642d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rbd19b3ee850444ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional Specs" sheetId="4" r:id="Rbb215e9051664201"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Components" sheetId="5" r:id="R6528b4b8ab9e4d69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification Inputs" sheetId="6" r:id="R4a88a93129ed4034"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Verification" sheetId="7" r:id="R34fdfe7f134a4029"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Verification" sheetId="8" r:id="R1eb5e5a782dd4a30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3-10 Verification" sheetId="9" r:id="R07d6a19c9c1a44b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v0.3.0 Traceability" sheetId="10" r:id="Rdb5d9cf260854225"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R1b4fb6db7b84491c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="2" r:id="R5ab766f0f5ae4bbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R168c6cc0af8748f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional Specs" sheetId="4" r:id="R61937d8273884b39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Components" sheetId="5" r:id="R2658dc137f5f496e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification Inputs" sheetId="6" r:id="R3cb1e1d172ca43aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Verification" sheetId="7" r:id="R7221a169bd1d47df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Verification" sheetId="8" r:id="R9b3b3145a02a40dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3-10 Verification" sheetId="9" r:id="R0ba27448f7414c54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v0.3.0 Traceability" sheetId="10" r:id="R14e1374f79d0475c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -86,7 +86,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="75">
+  <x:fills count="78">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -458,6 +458,21 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="6">
     <x:border/>
@@ -535,7 +550,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="206">
+  <x:cellXfs count="218">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1062,6 +1077,36 @@
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="74" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="75" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="76" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="75" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="77" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="77" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="75" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="76" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="76" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="76" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="77" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1458,7 +1503,7 @@
         <x:v>Design Components</x:v>
       </x:c>
       <x:c r="E5" s="9" t="n">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F5"/>
     </x:row>
@@ -1473,7 +1518,7 @@
         <x:v>Requirements with FS</x:v>
       </x:c>
       <x:c r="E6" s="9" t="n">
-        <x:v>138</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="F6"/>
     </x:row>
@@ -1482,13 +1527,13 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>0.5.0</x:v>
+        <x:v>0.6.0</x:v>
       </x:c>
       <x:c r="D7" s="11" t="str">
         <x:v>Requirements with Design</x:v>
       </x:c>
       <x:c r="E7" s="9" t="n">
-        <x:v>138</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="F7"/>
     </x:row>
@@ -1503,7 +1548,7 @@
         <x:v>Requirements with Verification</x:v>
       </x:c>
       <x:c r="E8" s="9" t="n">
-        <x:v>138</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="F8"/>
     </x:row>
@@ -1512,7 +1557,7 @@
         <x:v>Baseline Date</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-08-17</x:v>
+        <x:v>2026-08-20</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
         <x:v>Test Case IDs</x:v>
@@ -1526,13 +1571,13 @@
         <x:v>Normalized Requirements</x:v>
       </x:c>
       <x:c r="B10" s="9" t="n">
-        <x:v>138</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="D10" s="11" t="str">
         <x:v>Baseline Coverage</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>138 / 138 mapped</x:v>
+        <x:v>148 / 148 mapped</x:v>
       </x:c>
       <x:c r="F10"/>
     </x:row>
@@ -1541,7 +1586,7 @@
         <x:v>Functional Specifications</x:v>
       </x:c>
       <x:c r="B11" s="9" t="n">
-        <x:v>40</x:v>
+        <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1669,25 +1714,25 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="197" t="str">
+      <x:c r="A1" s="207" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="B1" s="197" t="str">
+      <x:c r="B1" s="207" t="str">
         <x:v>Functional Specification</x:v>
       </x:c>
-      <x:c r="C1" s="197" t="str">
+      <x:c r="C1" s="207" t="str">
         <x:v>Design</x:v>
       </x:c>
-      <x:c r="D1" s="197" t="str">
+      <x:c r="D1" s="207" t="str">
         <x:v>Implementation</x:v>
       </x:c>
-      <x:c r="E1" s="197" t="str">
+      <x:c r="E1" s="207" t="str">
         <x:v>Automated Verification</x:v>
       </x:c>
-      <x:c r="F1" s="197" t="str">
+      <x:c r="F1" s="207" t="str">
         <x:v>External Verification</x:v>
       </x:c>
-      <x:c r="G1" s="197" t="str">
+      <x:c r="G1" s="207" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -1710,7 +1755,7 @@
       <x:c r="F2" s="63" t="str">
         <x:v>EV-017</x:v>
       </x:c>
-      <x:c r="G2" s="199" t="str">
+      <x:c r="G2" s="209" t="str">
         <x:v>Auto PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -1733,7 +1778,7 @@
       <x:c r="F3" s="63" t="str">
         <x:v>EV-017</x:v>
       </x:c>
-      <x:c r="G3" s="199" t="str">
+      <x:c r="G3" s="209" t="str">
         <x:v>Auto PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -1756,7 +1801,7 @@
       <x:c r="F4" s="63" t="str">
         <x:v>EV-017</x:v>
       </x:c>
-      <x:c r="G4" s="199" t="str">
+      <x:c r="G4" s="209" t="str">
         <x:v>Static PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -1779,7 +1824,7 @@
       <x:c r="F5" s="63" t="str">
         <x:v>EV-018</x:v>
       </x:c>
-      <x:c r="G5" s="199" t="str">
+      <x:c r="G5" s="209" t="str">
         <x:v>Auto PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -1802,7 +1847,7 @@
       <x:c r="F6" s="63" t="str">
         <x:v>EV-018</x:v>
       </x:c>
-      <x:c r="G6" s="199" t="str">
+      <x:c r="G6" s="209" t="str">
         <x:v>Auto/Static PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -1825,7 +1870,7 @@
       <x:c r="F7" s="63" t="str">
         <x:v>EV-001</x:v>
       </x:c>
-      <x:c r="G7" s="199" t="str">
+      <x:c r="G7" s="209" t="str">
         <x:v>Auto PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -1848,7 +1893,7 @@
       <x:c r="F8" s="63" t="str">
         <x:v>EV-018</x:v>
       </x:c>
-      <x:c r="G8" s="199" t="str">
+      <x:c r="G8" s="209" t="str">
         <x:v>Auto/Static PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -1871,7 +1916,7 @@
       <x:c r="F9" s="63" t="str">
         <x:v>EV-017~EV-018</x:v>
       </x:c>
-      <x:c r="G9" s="199" t="str">
+      <x:c r="G9" s="209" t="str">
         <x:v>Auto PASS / External Pending</x:v>
       </x:c>
     </x:row>
@@ -5461,7 +5506,7 @@
         <x:v>REQ-IF-015</x:v>
       </x:c>
       <x:c r="B138" s="63" t="str">
-        <x:v>CAPL DLL Export Table은 Appendix A의 v0.5.0 23개 Entry를 정확히 제공하고 제거된 Monitoring·Change Queue API를 공개하지 않는다</x:v>
+        <x:v>CAPL DLL Export Table은 Appendix A의 v0.6.0 23개 Entry를 정확히 제공하고 제거된 Monitoring·Change Queue API를 공개하지 않는다</x:v>
       </x:c>
       <x:c r="C138" s="63" t="str">
         <x:v>FS-INIT-001; FS-MON-003; FS-DEVICE-001; FS-RTULOG-001</x:v>
@@ -5506,6 +5551,266 @@
       </x:c>
       <x:c r="H139" s="63" t="str">
         <x:v>IF-LIMIT-009; LOG-023~024; ERR-044</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A140" s="63" t="str">
+        <x:v>REQ-DPG-001</x:v>
+      </x:c>
+      <x:c r="B140" s="63" t="str">
+        <x:v>Device CSV와 각 CSV_DB_Name Register Map을 Core Loader 계약과 같은 Header·행·값·경로 규칙으로 분석하고 오류 파일/행/열/원인을 표시</x:v>
+      </x:c>
+      <x:c r="C140" s="63" t="str">
+        <x:v>FS-DPG-001</x:v>
+      </x:c>
+      <x:c r="D140" s="63" t="str">
+        <x:v>DC-20 Device Panel Generator</x:v>
+      </x:c>
+      <x:c r="E140" s="63" t="str">
+        <x:v>정상/오류 CSV fixture와 Core Loader 규칙 비교</x:v>
+      </x:c>
+      <x:c r="F140" s="63" t="str">
+        <x:v>TC-DPG-AUTO-001; EV-020</x:v>
+      </x:c>
+      <x:c r="G140" s="63" t="str">
+        <x:v>Automated PASS / External Pending</x:v>
+      </x:c>
+      <x:c r="H140" s="63" t="str">
+        <x:v>FR-DPG-001~003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A141" s="63" t="str">
+        <x:v>REQ-DPG-002</x:v>
+      </x:c>
+      <x:c r="B141" s="63" t="str">
+        <x:v>EXE 위치 기준 Output을 임시 경로에서 완전 생성·검증한 뒤 Manifest 소유 Output만 원자 교체하고 동일 입력은 byte-identical 결과를 생성</x:v>
+      </x:c>
+      <x:c r="C141" s="63" t="str">
+        <x:v>FS-DPG-001</x:v>
+      </x:c>
+      <x:c r="D141" s="63" t="str">
+        <x:v>DC-20 Device Panel Generator</x:v>
+      </x:c>
+      <x:c r="E141" s="63" t="str">
+        <x:v>deterministic output, transaction rollback, manifest guard와 다른 cwd EXE smoke</x:v>
+      </x:c>
+      <x:c r="F141" s="63" t="str">
+        <x:v>TC-DPG-AUTO-001; EV-020</x:v>
+      </x:c>
+      <x:c r="G141" s="63" t="str">
+        <x:v>Automated PASS / External Pending</x:v>
+      </x:c>
+      <x:c r="H141" s="63" t="str">
+        <x:v>FR-DPG-004~005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A142" s="63" t="str">
+        <x:v>REQ-DPG-003</x:v>
+      </x:c>
+      <x:c r="B142" s="63" t="str">
+        <x:v>실제 Device Index와 Decimal Address 31-register Group, 15행 Page로 독립 XVP Fragment를 만들고 고유 Object/Control/TabIndex와 정확한 바인딩을 제공</x:v>
+      </x:c>
+      <x:c r="C142" s="63" t="str">
+        <x:v>FS-DPG-002</x:v>
+      </x:c>
+      <x:c r="D142" s="63" t="str">
+        <x:v>DC-20 Device Panel Generator</x:v>
+      </x:c>
+      <x:c r="E142" s="63" t="str">
+        <x:v>34/45/72/150 Signal XVP XML·Address group·page·binding 검사</x:v>
+      </x:c>
+      <x:c r="F142" s="63" t="str">
+        <x:v>TC-DPG-AUTO-001; EV-020</x:v>
+      </x:c>
+      <x:c r="G142" s="63" t="str">
+        <x:v>Automated PASS / External Pending</x:v>
+      </x:c>
+      <x:c r="H142" s="63" t="str">
+        <x:v>FR-DPG-006~009</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A143" s="63" t="str">
+        <x:v>REQ-DPG-004</x:v>
+      </x:c>
+      <x:c r="B143" s="63" t="str">
+        <x:v>Common 및 Device별 PhysicalValue/RawHex/Command/Snapshot/Result System Variable 계약을 생성하고 각 Device baseline과 결과를 격리</x:v>
+      </x:c>
+      <x:c r="C143" s="63" t="str">
+        <x:v>FS-DPG-002</x:v>
+      </x:c>
+      <x:c r="D143" s="63" t="str">
+        <x:v>DC-20 Generator; DC-21 Generated CAPL</x:v>
+      </x:c>
+      <x:c r="E143" s="63" t="str">
+        <x:v>vsysvar schema와 sample generated artifact stale 검사</x:v>
+      </x:c>
+      <x:c r="F143" s="63" t="str">
+        <x:v>TC-DPG-AUTO-001; EV-020</x:v>
+      </x:c>
+      <x:c r="G143" s="63" t="str">
+        <x:v>Automated/Static PASS / External Pending</x:v>
+      </x:c>
+      <x:c r="H143" s="63" t="str">
+        <x:v>FR-DPG-010</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A144" s="63" t="str">
+        <x:v>REQ-DPG-005</x:v>
+      </x:c>
+      <x:c r="B144" s="63" t="str">
+        <x:v>Raw Hex는 정규화 논리 Signal Frame에서 Start_Bit/Size로 추출한 1~64bit unsigned pattern을 대문자·leading zero로 표시하고 frame 공유 Signal은 Register Read를 재사용</x:v>
+      </x:c>
+      <x:c r="C144" s="63" t="str">
+        <x:v>FS-DPG-003</x:v>
+      </x:c>
+      <x:c r="D144" s="63" t="str">
+        <x:v>DC-21 Generated Device Panel CAPL</x:v>
+      </x:c>
+      <x:c r="E144" s="63" t="str">
+        <x:v>1~64bit, endian, bit crossing, signed/float/double/full-range raw vectors</x:v>
+      </x:c>
+      <x:c r="F144" s="63" t="str">
+        <x:v>TC-DPG-AUTO-001; EV-020</x:v>
+      </x:c>
+      <x:c r="G144" s="63" t="str">
+        <x:v>Automated/Static PASS / External Pending</x:v>
+      </x:c>
+      <x:c r="H144" s="63" t="str">
+        <x:v>FR-DPG-011~012</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A145" s="63" t="str">
+        <x:v>REQ-DPG-006</x:v>
+      </x:c>
+      <x:c r="B145" s="63" t="str">
+        <x:v>Display Update는 15 Signal bounded timer chunk로 Physical/Raw를 요청 시에만 읽고 성공한 전체 결과만 baseline/SnapshotValid로 게시하며 재진입을 Busy로 거부</x:v>
+      </x:c>
+      <x:c r="C145" s="63" t="str">
+        <x:v>FS-DPG-003</x:v>
+      </x:c>
+      <x:c r="D145" s="63" t="str">
+        <x:v>DC-21 Generated Device Panel CAPL</x:v>
+      </x:c>
+      <x:c r="E145" s="63" t="str">
+        <x:v>chunk/busy/snapshot/raw stale-clear CAPL source contract</x:v>
+      </x:c>
+      <x:c r="F145" s="63" t="str">
+        <x:v>TC-DPG-AUTO-001; EV-020</x:v>
+      </x:c>
+      <x:c r="G145" s="63" t="str">
+        <x:v>Static PASS / External Pending</x:v>
+      </x:c>
+      <x:c r="H145" s="63" t="str">
+        <x:v>FR-DPG-013</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A146" s="63" t="str">
+        <x:v>REQ-DPG-007</x:v>
+      </x:c>
+      <x:c r="B146" s="63" t="str">
+        <x:v>Send Changed는 유효 Snapshot baseline과 다른 Signal만 CSV 순서로 Write하고 첫 실패에서 중단하며 성공 Signal read-back·양자화·결과를 반영</x:v>
+      </x:c>
+      <x:c r="C146" s="63" t="str">
+        <x:v>FS-DPG-004</x:v>
+      </x:c>
+      <x:c r="D146" s="63" t="str">
+        <x:v>DC-21 Generated Device Panel CAPL</x:v>
+      </x:c>
+      <x:c r="E146" s="63" t="str">
+        <x:v>baseline compare, ordered partial send, read-back/result source contract</x:v>
+      </x:c>
+      <x:c r="F146" s="63" t="str">
+        <x:v>TC-DPG-AUTO-001; EV-020</x:v>
+      </x:c>
+      <x:c r="G146" s="63" t="str">
+        <x:v>Static PASS / External Pending</x:v>
+      </x:c>
+      <x:c r="H146" s="63" t="str">
+        <x:v>FR-DPG-014</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A147" s="63" t="str">
+        <x:v>REQ-DPG-008</x:v>
+      </x:c>
+      <x:c r="B147" s="63" t="str">
+        <x:v>Device Reset은 ResetDevice 후 read-back하고 Reset All은 실제 Index 오름차순으로 비원자 처리해 완료 수·첫 실패 Index·Result를 게시</x:v>
+      </x:c>
+      <x:c r="C147" s="63" t="str">
+        <x:v>FS-DPG-004</x:v>
+      </x:c>
+      <x:c r="D147" s="63" t="str">
+        <x:v>DC-21 Generated Device Panel CAPL</x:v>
+      </x:c>
+      <x:c r="E147" s="63" t="str">
+        <x:v>momentary reset, ascending sparse Index reset-all/result source contract</x:v>
+      </x:c>
+      <x:c r="F147" s="63" t="str">
+        <x:v>TC-DPG-AUTO-001; EV-020</x:v>
+      </x:c>
+      <x:c r="G147" s="63" t="str">
+        <x:v>Static PASS / External Pending</x:v>
+      </x:c>
+      <x:c r="H147" s="63" t="str">
+        <x:v>FR-DPG-015~016</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A148" s="63" t="str">
+        <x:v>REQ-DPG-009</x:v>
+      </x:c>
+      <x:c r="B148" s="63" t="str">
+        <x:v>Refresh 성공 시 모든 Snapshot을 무효화하고 Display Update가 Device 전체 동일시점 Snapshot이 아니며 Send/Reset All이 전체 Transaction 원자적이지 않음을 보존·표시</x:v>
+      </x:c>
+      <x:c r="C148" s="63" t="str">
+        <x:v>FS-DPG-004</x:v>
+      </x:c>
+      <x:c r="D148" s="63" t="str">
+        <x:v>DC-21 Generated Device Panel CAPL</x:v>
+      </x:c>
+      <x:c r="E148" s="63" t="str">
+        <x:v>Refresh 성공 invalidate, busy와 비원자 경계 정적/외부 시험</x:v>
+      </x:c>
+      <x:c r="F148" s="63" t="str">
+        <x:v>TC-DPG-AUTO-001; EV-020</x:v>
+      </x:c>
+      <x:c r="G148" s="63" t="str">
+        <x:v>Static PASS / External Pending</x:v>
+      </x:c>
+      <x:c r="H148" s="63" t="str">
+        <x:v>FR-DPG-017~019</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A149" s="63" t="str">
+        <x:v>REQ-DPG-010</x:v>
+      </x:c>
+      <x:c r="B149" s="63" t="str">
+        <x:v>PyInstaller one-file Generator, Sample generated Config, Manifest/COPY_GUIDE와 회사 적용·재생성 절차를 배포하며 실제 회사 Map을 저장소에 포함하지 않음</x:v>
+      </x:c>
+      <x:c r="C149" s="63" t="str">
+        <x:v>FS-DPG-005</x:v>
+      </x:c>
+      <x:c r="D149" s="63" t="str">
+        <x:v>DC-20 Device Panel Generator</x:v>
+      </x:c>
+      <x:c r="E149" s="63" t="str">
+        <x:v>one-file EXE, portable package, COPY_GUIDE, manifest/hash 검사</x:v>
+      </x:c>
+      <x:c r="F149" s="63" t="str">
+        <x:v>TC-DPG-AUTO-001; EV-020</x:v>
+      </x:c>
+      <x:c r="G149" s="63" t="str">
+        <x:v>Automated PASS / External Pending</x:v>
+      </x:c>
+      <x:c r="H149" s="63" t="str">
+        <x:v>FR-DPG-020</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5516,7 +5821,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5c26bf976754e3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R355494b01d764169"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8693,7 +8998,7 @@
         <x:v>API</x:v>
       </x:c>
       <x:c r="C138" s="63" t="str">
-        <x:v>CAPL DLL Export Table은 Appendix A의 v0.5.0 23개 Entry를 정확히 제공하고 제거된 Monitoring·Change Queue API를 공개하지 않는다</x:v>
+        <x:v>CAPL DLL Export Table은 Appendix A의 v0.6.0 23개 Entry를 정확히 제공하고 제거된 Monitoring·Change Queue API를 공개하지 않는다</x:v>
       </x:c>
       <x:c r="D138" s="63" t="str">
         <x:v>IF-API-001~008; IF-API-011; IF-API-014~027; COMP-009</x:v>
@@ -8731,10 +9036,240 @@
         <x:v>Queue 경계·overflow·idle wake/timeout·pair 보존 자동 시험과 EV-018</x:v>
       </x:c>
     </x:row>
+    <x:row r="140" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A140" s="63" t="str">
+        <x:v>REQ-DPG-001</x:v>
+      </x:c>
+      <x:c r="B140" s="63" t="str">
+        <x:v>Generator</x:v>
+      </x:c>
+      <x:c r="C140" s="63" t="str">
+        <x:v>Device CSV와 각 CSV_DB_Name Register Map을 Core Loader 계약과 같은 Header·행·값·경로 규칙으로 분석하고 오류 파일/행/열/원인을 표시</x:v>
+      </x:c>
+      <x:c r="D140" s="63" t="str">
+        <x:v>FR-DPG-001~003</x:v>
+      </x:c>
+      <x:c r="E140" s="63" t="str">
+        <x:v>FS-DPG-001</x:v>
+      </x:c>
+      <x:c r="F140" s="63" t="str">
+        <x:v>DC-20</x:v>
+      </x:c>
+      <x:c r="G140" s="63" t="str">
+        <x:v>Python 자동시험과 EV-020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A141" s="63" t="str">
+        <x:v>REQ-DPG-002</x:v>
+      </x:c>
+      <x:c r="B141" s="63" t="str">
+        <x:v>Generator</x:v>
+      </x:c>
+      <x:c r="C141" s="63" t="str">
+        <x:v>EXE 위치 기준 Output을 임시 경로에서 완전 생성·검증한 뒤 Manifest 소유 Output만 원자 교체하고 동일 입력은 byte-identical 결과를 생성</x:v>
+      </x:c>
+      <x:c r="D141" s="63" t="str">
+        <x:v>FR-DPG-004~005</x:v>
+      </x:c>
+      <x:c r="E141" s="63" t="str">
+        <x:v>FS-DPG-001</x:v>
+      </x:c>
+      <x:c r="F141" s="63" t="str">
+        <x:v>DC-20</x:v>
+      </x:c>
+      <x:c r="G141" s="63" t="str">
+        <x:v>transaction·determinism·manifest guard·다른 cwd EXE 시험과 EV-020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A142" s="63" t="str">
+        <x:v>REQ-DPG-003</x:v>
+      </x:c>
+      <x:c r="B142" s="63" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="C142" s="63" t="str">
+        <x:v>실제 Device Index와 Decimal Address 31-register Group, 15행 Page로 독립 XVP Fragment를 만들고 고유 Object/Control/TabIndex와 정확한 바인딩을 제공</x:v>
+      </x:c>
+      <x:c r="D142" s="63" t="str">
+        <x:v>FR-DPG-006~009</x:v>
+      </x:c>
+      <x:c r="E142" s="63" t="str">
+        <x:v>FS-DPG-002</x:v>
+      </x:c>
+      <x:c r="F142" s="63" t="str">
+        <x:v>DC-20</x:v>
+      </x:c>
+      <x:c r="G142" s="63" t="str">
+        <x:v>XVP XML·GroupBox·page·binding 자동시험과 EV-020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A143" s="63" t="str">
+        <x:v>REQ-DPG-004</x:v>
+      </x:c>
+      <x:c r="B143" s="63" t="str">
+        <x:v>Interface</x:v>
+      </x:c>
+      <x:c r="C143" s="63" t="str">
+        <x:v>Common 및 Device별 PhysicalValue/RawHex/Command/Snapshot/Result System Variable 계약을 생성하고 각 Device baseline과 결과를 격리</x:v>
+      </x:c>
+      <x:c r="D143" s="63" t="str">
+        <x:v>FR-DPG-010</x:v>
+      </x:c>
+      <x:c r="E143" s="63" t="str">
+        <x:v>FS-DPG-002</x:v>
+      </x:c>
+      <x:c r="F143" s="63" t="str">
+        <x:v>DC-20; DC-21</x:v>
+      </x:c>
+      <x:c r="G143" s="63" t="str">
+        <x:v>generated vsysvar stale/source contract와 EV-020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A144" s="63" t="str">
+        <x:v>REQ-DPG-005</x:v>
+      </x:c>
+      <x:c r="B144" s="63" t="str">
+        <x:v>Data</x:v>
+      </x:c>
+      <x:c r="C144" s="63" t="str">
+        <x:v>Raw Hex는 정규화 논리 Signal Frame에서 Start_Bit/Size로 추출한 1~64bit unsigned pattern을 대문자·leading zero로 표시하고 frame 공유 Signal은 Register Read를 재사용</x:v>
+      </x:c>
+      <x:c r="D144" s="63" t="str">
+        <x:v>FR-DPG-011~012</x:v>
+      </x:c>
+      <x:c r="E144" s="63" t="str">
+        <x:v>FS-DPG-003</x:v>
+      </x:c>
+      <x:c r="F144" s="63" t="str">
+        <x:v>DC-21</x:v>
+      </x:c>
+      <x:c r="G144" s="63" t="str">
+        <x:v>Endian/bit/nibble/frame-cache vector 자동시험과 EV-020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A145" s="63" t="str">
+        <x:v>REQ-DPG-006</x:v>
+      </x:c>
+      <x:c r="B145" s="63" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="C145" s="63" t="str">
+        <x:v>Display Update는 15 Signal bounded timer chunk로 Physical/Raw를 요청 시에만 읽고 성공한 전체 결과만 baseline/SnapshotValid로 게시하며 재진입을 Busy로 거부</x:v>
+      </x:c>
+      <x:c r="D145" s="63" t="str">
+        <x:v>FR-DPG-013</x:v>
+      </x:c>
+      <x:c r="E145" s="63" t="str">
+        <x:v>FS-DPG-003</x:v>
+      </x:c>
+      <x:c r="F145" s="63" t="str">
+        <x:v>DC-21</x:v>
+      </x:c>
+      <x:c r="G145" s="63" t="str">
+        <x:v>generated CAPL source contract와 EV-020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A146" s="63" t="str">
+        <x:v>REQ-DPG-007</x:v>
+      </x:c>
+      <x:c r="B146" s="63" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="C146" s="63" t="str">
+        <x:v>Send Changed는 유효 Snapshot baseline과 다른 Signal만 CSV 순서로 Write하고 첫 실패에서 중단하며 성공 Signal read-back·양자화·결과를 반영</x:v>
+      </x:c>
+      <x:c r="D146" s="63" t="str">
+        <x:v>FR-DPG-014</x:v>
+      </x:c>
+      <x:c r="E146" s="63" t="str">
+        <x:v>FS-DPG-004</x:v>
+      </x:c>
+      <x:c r="F146" s="63" t="str">
+        <x:v>DC-21</x:v>
+      </x:c>
+      <x:c r="G146" s="63" t="str">
+        <x:v>generated CAPL source contract와 EV-020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A147" s="63" t="str">
+        <x:v>REQ-DPG-008</x:v>
+      </x:c>
+      <x:c r="B147" s="63" t="str">
+        <x:v>Panel</x:v>
+      </x:c>
+      <x:c r="C147" s="63" t="str">
+        <x:v>Device Reset은 ResetDevice 후 read-back하고 Reset All은 실제 Index 오름차순으로 비원자 처리해 완료 수·첫 실패 Index·Result를 게시</x:v>
+      </x:c>
+      <x:c r="D147" s="63" t="str">
+        <x:v>FR-DPG-015~016</x:v>
+      </x:c>
+      <x:c r="E147" s="63" t="str">
+        <x:v>FS-DPG-004</x:v>
+      </x:c>
+      <x:c r="F147" s="63" t="str">
+        <x:v>DC-21</x:v>
+      </x:c>
+      <x:c r="G147" s="63" t="str">
+        <x:v>generated CAPL source contract와 EV-020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A148" s="63" t="str">
+        <x:v>REQ-DPG-009</x:v>
+      </x:c>
+      <x:c r="B148" s="63" t="str">
+        <x:v>Concurrency</x:v>
+      </x:c>
+      <x:c r="C148" s="63" t="str">
+        <x:v>Refresh 성공 시 모든 Snapshot을 무효화하고 Display Update가 Device 전체 동일시점 Snapshot이 아니며 Send/Reset All이 전체 Transaction 원자적이지 않음을 보존·표시</x:v>
+      </x:c>
+      <x:c r="D148" s="63" t="str">
+        <x:v>FR-DPG-017~019</x:v>
+      </x:c>
+      <x:c r="E148" s="63" t="str">
+        <x:v>FS-DPG-004</x:v>
+      </x:c>
+      <x:c r="F148" s="63" t="str">
+        <x:v>DC-21</x:v>
+      </x:c>
+      <x:c r="G148" s="63" t="str">
+        <x:v>refresh/busy/non-atomic source contract와 EV-020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A149" s="63" t="str">
+        <x:v>REQ-DPG-010</x:v>
+      </x:c>
+      <x:c r="B149" s="63" t="str">
+        <x:v>Release</x:v>
+      </x:c>
+      <x:c r="C149" s="63" t="str">
+        <x:v>PyInstaller one-file Generator, Sample generated Config, Manifest/COPY_GUIDE와 회사 적용·재생성 절차를 배포하며 실제 회사 Map을 저장소에 포함하지 않음</x:v>
+      </x:c>
+      <x:c r="D149" s="63" t="str">
+        <x:v>FR-DPG-020</x:v>
+      </x:c>
+      <x:c r="E149" s="63" t="str">
+        <x:v>FS-DPG-005</x:v>
+      </x:c>
+      <x:c r="F149" s="63" t="str">
+        <x:v>DC-20</x:v>
+      </x:c>
+      <x:c r="G149" s="63" t="str">
+        <x:v>EXE/package/hash 자동시험과 EV-020</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a0611f3cc0146a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R213a7c266a614990"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9199,10 +9734,65 @@
         <x:v>REQ-FUNC-048~049; REQ-IF-015~016</x:v>
       </x:c>
     </x:row>
+    <x:row r="42" ht="15" hidden="0" customHeight="1">
+      <x:c r="A42" s="63" t="str">
+        <x:v>FS-DPG-001</x:v>
+      </x:c>
+      <x:c r="B42" s="63" t="str">
+        <x:v>Device/Register CSV 분석과 Transaction 생성</x:v>
+      </x:c>
+      <x:c r="C42" s="63" t="str">
+        <x:v>REQ-DPG-001~002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="15" hidden="0" customHeight="1">
+      <x:c r="A43" s="63" t="str">
+        <x:v>FS-DPG-002</x:v>
+      </x:c>
+      <x:c r="B43" s="63" t="str">
+        <x:v>XVP Fragment와 System Variable DB 생성</x:v>
+      </x:c>
+      <x:c r="C43" s="63" t="str">
+        <x:v>REQ-DPG-003~004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="15" hidden="0" customHeight="1">
+      <x:c r="A44" s="63" t="str">
+        <x:v>FS-DPG-003</x:v>
+      </x:c>
+      <x:c r="B44" s="63" t="str">
+        <x:v>Raw Hex와 bounded Display Update</x:v>
+      </x:c>
+      <x:c r="C44" s="63" t="str">
+        <x:v>REQ-DPG-005~006</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="15" hidden="0" customHeight="1">
+      <x:c r="A45" s="63" t="str">
+        <x:v>FS-DPG-004</x:v>
+      </x:c>
+      <x:c r="B45" s="63" t="str">
+        <x:v>Send Changed와 Device/All Reset</x:v>
+      </x:c>
+      <x:c r="C45" s="63" t="str">
+        <x:v>REQ-DPG-007~009</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="15" hidden="0" customHeight="1">
+      <x:c r="A46" s="63" t="str">
+        <x:v>FS-DPG-005</x:v>
+      </x:c>
+      <x:c r="B46" s="63" t="str">
+        <x:v>Python-free 배포와 회사 적용 절차</x:v>
+      </x:c>
+      <x:c r="C46" s="63" t="str">
+        <x:v>REQ-DPG-010</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R343186bef1974b68"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96ff1c0519b84583"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9436,10 +10026,32 @@
         <x:v>PortWorker 관측점, Transaction Queue, REQ/RES·NO_RES pairing, CAPL-only 전체 CSV Writer와 동일 Drain 문자열의 최근 10줄·200ms Output View</x:v>
       </x:c>
     </x:row>
+    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A21" s="63" t="str">
+        <x:v>DC-20</x:v>
+      </x:c>
+      <x:c r="B21" s="63" t="str">
+        <x:v>Device Panel Generator</x:v>
+      </x:c>
+      <x:c r="C21" s="63" t="str">
+        <x:v>Python stdlib/tkinter GUI·CLI 공통 Parser/Generator, XVP·vsysvar·CAPL·Manifest Transaction 출력, PyInstaller one-file</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A22" s="63" t="str">
+        <x:v>DC-21</x:v>
+      </x:c>
+      <x:c r="B22" s="63" t="str">
+        <x:v>Generated Device Panel CAPL</x:v>
+      </x:c>
+      <x:c r="C22" s="63" t="str">
+        <x:v>M485E_UI include 체계, Device별 bounded timer 작업·baseline·Raw Hex frame cache·SnapshotValid·momentary command adapter</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R941f46324778426f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R671cbb1101a8456b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9546,7 +10158,7 @@
         <x:v>External Test Result</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>19건 Not Tested</x:v>
+        <x:v>20건 Not Tested</x:v>
       </x:c>
       <x:c r="C9" t="str">
         <x:v>docs/05_Test/Modbus485Emulator_External_Test_Result.xlsx</x:v>
@@ -9577,7 +10189,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bdaeff5f72c40fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R761729bb63a04af6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9884,7 +10496,7 @@
       <x:c r="D7" s="35" t="str">
         <x:v>CANalyzer 13 x86</x:v>
       </x:c>
-      <x:c r="E7" s="196" t="str">
+      <x:c r="E7" s="206" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F7" s="35" t="str">
@@ -9930,25 +10542,25 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="197" t="str">
+      <x:c r="A1" s="207" t="str">
         <x:v>Test Case ID</x:v>
       </x:c>
-      <x:c r="B1" s="197" t="str">
+      <x:c r="B1" s="207" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="C1" s="197" t="str">
+      <x:c r="C1" s="207" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="D1" s="197" t="str">
+      <x:c r="D1" s="207" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="E1" s="197" t="str">
+      <x:c r="E1" s="207" t="str">
         <x:v>Method</x:v>
       </x:c>
-      <x:c r="F1" s="197" t="str">
+      <x:c r="F1" s="207" t="str">
         <x:v>Result</x:v>
       </x:c>
-      <x:c r="G1" s="197" t="str">
+      <x:c r="G1" s="207" t="str">
         <x:v>External Follow-up</x:v>
       </x:c>
     </x:row>
@@ -9968,7 +10580,7 @@
       <x:c r="E2" s="63" t="str">
         <x:v>M485E.Core.Tests</x:v>
       </x:c>
-      <x:c r="F2" s="198" t="str">
+      <x:c r="F2" s="208" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G2" s="63" t="str">
@@ -9991,7 +10603,7 @@
       <x:c r="E3" s="63" t="str">
         <x:v>M485E.Core.Tests</x:v>
       </x:c>
-      <x:c r="F3" s="198" t="str">
+      <x:c r="F3" s="208" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G3" s="63" t="str">
@@ -10014,7 +10626,7 @@
       <x:c r="E4" s="63" t="str">
         <x:v>M485E.Core.Tests</x:v>
       </x:c>
-      <x:c r="F4" s="198" t="str">
+      <x:c r="F4" s="208" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G4" s="63" t="str">
@@ -10037,7 +10649,7 @@
       <x:c r="E5" s="63" t="str">
         <x:v>M485E.Core.Tests</x:v>
       </x:c>
-      <x:c r="F5" s="198" t="str">
+      <x:c r="F5" s="208" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G5" s="63" t="str">
@@ -10060,7 +10672,7 @@
       <x:c r="E6" s="63" t="str">
         <x:v>M485E.Core.Tests + FakeSerialTransport</x:v>
       </x:c>
-      <x:c r="F6" s="198" t="str">
+      <x:c r="F6" s="208" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G6" s="63" t="str">
@@ -10083,7 +10695,7 @@
       <x:c r="E7" s="63" t="str">
         <x:v>M485E.IntegrationTests</x:v>
       </x:c>
-      <x:c r="F7" s="198" t="str">
+      <x:c r="F7" s="208" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G7" s="63" t="str">
@@ -10106,7 +10718,7 @@
       <x:c r="E8" s="63" t="str">
         <x:v>Test-M485ECaplSources.ps1 + CANalyzer 13 Exec32 caplcompexec</x:v>
       </x:c>
-      <x:c r="F8" s="198" t="str">
+      <x:c r="F8" s="208" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G8" s="63" t="str">
@@ -10129,7 +10741,7 @@
       <x:c r="E9" s="63" t="str">
         <x:v>Test-M485ECaplSources.ps1; Main compile in configured CANalyzer project</x:v>
       </x:c>
-      <x:c r="F9" s="199" t="str">
+      <x:c r="F9" s="209" t="str">
         <x:v>Static PASS / External Pending</x:v>
       </x:c>
       <x:c r="G9" s="63" t="str">
@@ -10152,7 +10764,7 @@
       <x:c r="E10" s="63" t="str">
         <x:v>MSBuild + CMake + CTest + CANalyzer 13 x86 CAPL compiler</x:v>
       </x:c>
-      <x:c r="F10" s="198" t="str">
+      <x:c r="F10" s="208" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G10" s="63" t="str">
@@ -10175,56 +10787,79 @@
       <x:c r="E11" s="63" t="str">
         <x:v>M485E.Core.Tests + M485E.IntegrationTests + Test-M485ECaplSources.ps1</x:v>
       </x:c>
-      <x:c r="F11" s="199" t="str">
+      <x:c r="F11" s="209" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="G11" s="63" t="str">
         <x:v>EV-017~EV-019</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="12" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A12" s="63" t="str">
-        <x:v>EV-001~EV-019</x:v>
+        <x:v>TC-DPG-AUTO-001</x:v>
       </x:c>
       <x:c r="B12" s="63" t="str">
-        <x:v>External</x:v>
+        <x:v>10/11</x:v>
       </x:c>
       <x:c r="C12" s="63" t="str">
-        <x:v>External</x:v>
+        <x:v>Automated + Static</x:v>
       </x:c>
       <x:c r="D12" s="63" t="str">
-        <x:v>CANalyzer 9.x/18, SystemBase Multi USB-485, Board, Panel, CAPL Output View, virtual CAN, RTU CSV</x:v>
+        <x:v>CSV 계약·경로 안전성·deterministic transaction 출력, XVP XML/바인딩, Raw Hex vectors, generated CAPL/vsysvar stale, one-file EXE 다른 cwd smoke</x:v>
       </x:c>
       <x:c r="E12" s="63" t="str">
-        <x:v>External Verification Guide</x:v>
-      </x:c>
-      <x:c r="F12" s="198" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Python unittest + Test-M485EDevicePanelSources.ps1 + Test-PanelGeneratorExe.ps1</x:v>
+      </x:c>
+      <x:c r="F12" s="209" t="str">
+        <x:v>PASS / External Pending</x:v>
       </x:c>
       <x:c r="G12" s="63" t="str">
-        <x:v>대상 실환경에서 결과 기록</x:v>
+        <x:v>EV-020</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A13" s="63" t="str">
+        <x:v>EV-001~EV-020</x:v>
+      </x:c>
+      <x:c r="B13" s="63" t="str">
+        <x:v>External</x:v>
+      </x:c>
+      <x:c r="C13" s="63" t="str">
+        <x:v>External</x:v>
+      </x:c>
+      <x:c r="D13" s="63" t="str">
+        <x:v>CANalyzer 9.x/18, SystemBase Multi USB-485, Board, Panel/XVP copy, CAPL Output View, virtual CAN, RTU CSV</x:v>
+      </x:c>
+      <x:c r="E13" s="63" t="str">
+        <x:v>External Verification Guide</x:v>
+      </x:c>
+      <x:c r="F13" s="209" t="str">
+        <x:v>Not Tested</x:v>
+      </x:c>
+      <x:c r="G13" s="63" t="str">
+        <x:v>대상 실환경에서 결과 기록</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A14" s="63" t="str">
         <x:v>TC-CAPL13-COMPILE-001</x:v>
       </x:c>
-      <x:c r="B13" s="63" t="str">
+      <x:c r="B14" s="63" t="str">
         <x:v>1/2/9</x:v>
       </x:c>
-      <x:c r="C13" s="63" t="str">
+      <x:c r="C14" s="63" t="str">
         <x:v>Compiler</x:v>
       </x:c>
-      <x:c r="D13" s="63" t="str">
+      <x:c r="D14" s="63" t="str">
         <x:v>Phase 1 ABI, Phase 2 Contracts, Phase 9 Core/Monitoring CAPL probes</x:v>
       </x:c>
-      <x:c r="E13" s="63" t="str">
+      <x:c r="E14" s="63" t="str">
         <x:v>CANalyzer 13 Exec32 caplcompexec.exe</x:v>
       </x:c>
-      <x:c r="F13" s="198" t="str">
+      <x:c r="F14" s="208" t="str">
         <x:v>PASS (warning-free)</x:v>
       </x:c>
-      <x:c r="G13" s="63" t="str">
+      <x:c r="G14" s="63" t="str">
         <x:v>CANalyzer 9.x SP8 Compile/Measurement remains EV-001</x:v>
       </x:c>
     </x:row>

</xml_diff>